<commit_message>
Update MLB weather 2026-07-16 09:24 PM PT
</commit_message>
<xml_diff>
--- a/mlb_weather_professional_v4_2026_07_17.xlsx
+++ b/mlb_weather_professional_v4_2026_07_17.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1852" uniqueCount="366">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1852" uniqueCount="364">
   <si>
     <t>Date</t>
   </si>
@@ -587,49 +587,46 @@
     <t>MEDIUM</t>
   </si>
   <si>
-    <t>2026-07-16 09:17:48 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-16 09:17:49 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-16 09:17:50 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-16 09:17:51 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-16 09:17:53 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-16 09:17:57 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-16 09:17:59 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-16 09:18:00 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-16 09:18:01 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-16 09:18:03 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-16 09:18:04 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-16 09:18:05 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-16 09:18:06 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-16 09:18:08 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-16 09:18:09 PM PDT</t>
+    <t>2026-07-16 09:24:25 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-16 09:24:26 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-16 09:24:27 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-16 09:24:28 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-16 09:24:29 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-16 09:24:33 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-16 09:24:34 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-16 09:24:35 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-16 09:24:36 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-16 09:24:37 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-16 09:24:38 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-16 09:24:39 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-16 09:24:40 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-16 09:24:41 PM PDT</t>
   </si>
   <si>
     <t>Period</t>
@@ -962,49 +959,46 @@
     <t>10:10 PM PDT</t>
   </si>
   <si>
-    <t>2026-07-17 04:17:48 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-17 04:17:49 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-17 04:17:50 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-17 04:17:51 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-17 04:17:53 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-17 04:17:57 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-17 04:17:59 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-17 04:18:00 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-17 04:18:01 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-17 04:18:03 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-17 04:18:04 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-17 04:18:05 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-17 04:18:06 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-17 04:18:08 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-17 04:18:09 UTC</t>
+    <t>2026-07-17 04:24:25 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-17 04:24:26 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-17 04:24:27 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-17 04:24:28 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-17 04:24:29 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-17 04:24:33 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-17 04:24:34 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-17 04:24:35 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-17 04:24:36 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-17 04:24:37 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-17 04:24:38 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-17 04:24:39 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-17 04:24:40 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-17 04:24:41 UTC</t>
   </si>
   <si>
     <t>2026-07-16T19:01:48+00:00</t>
@@ -1919,7 +1913,7 @@
         <v>188</v>
       </c>
       <c r="AY2">
-        <v>556</v>
+        <v>562.6</v>
       </c>
       <c r="AZ2">
         <v>5</v>
@@ -2074,7 +2068,7 @@
         <v>189</v>
       </c>
       <c r="AY3">
-        <v>336.4</v>
+        <v>343</v>
       </c>
       <c r="AZ3">
         <v>5</v>
@@ -2229,7 +2223,7 @@
         <v>190</v>
       </c>
       <c r="AY4">
-        <v>556</v>
+        <v>562.7</v>
       </c>
       <c r="AZ4">
         <v>5</v>
@@ -2384,7 +2378,7 @@
         <v>191</v>
       </c>
       <c r="AY5">
-        <v>481.2</v>
+        <v>487.8</v>
       </c>
       <c r="AZ5">
         <v>5</v>
@@ -2515,7 +2509,7 @@
         <v>183</v>
       </c>
       <c r="AQ6">
-        <v>8.1</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="AR6">
         <v>0</v>
@@ -2539,7 +2533,7 @@
         <v>192</v>
       </c>
       <c r="AY6">
-        <v>325.3</v>
+        <v>331.9</v>
       </c>
       <c r="AZ6">
         <v>5</v>
@@ -2670,7 +2664,7 @@
         <v>183</v>
       </c>
       <c r="AQ7">
-        <v>5.1</v>
+        <v>5.6</v>
       </c>
       <c r="AR7">
         <v>0</v>
@@ -2849,7 +2843,7 @@
         <v>194</v>
       </c>
       <c r="AY8">
-        <v>160.7</v>
+        <v>167.3</v>
       </c>
       <c r="AZ8">
         <v>5</v>
@@ -3004,7 +2998,7 @@
         <v>195</v>
       </c>
       <c r="AY9">
-        <v>56.6</v>
+        <v>63.2</v>
       </c>
       <c r="AZ9">
         <v>5</v>
@@ -3159,7 +3153,7 @@
         <v>196</v>
       </c>
       <c r="AY10">
-        <v>31.6</v>
+        <v>38.2</v>
       </c>
       <c r="AZ10">
         <v>5</v>
@@ -3290,7 +3284,7 @@
         <v>183</v>
       </c>
       <c r="AQ11">
-        <v>12.9</v>
+        <v>13.5</v>
       </c>
       <c r="AR11">
         <v>0</v>
@@ -3314,7 +3308,7 @@
         <v>197</v>
       </c>
       <c r="AY11">
-        <v>5.9</v>
+        <v>12.4</v>
       </c>
       <c r="AZ11">
         <v>5</v>
@@ -3469,7 +3463,7 @@
         <v>198</v>
       </c>
       <c r="AY12">
-        <v>571.6</v>
+        <v>578.2</v>
       </c>
       <c r="AZ12">
         <v>5</v>
@@ -3555,7 +3549,7 @@
         <v>2.2</v>
       </c>
       <c r="AB13">
-        <v>90.09999999999999</v>
+        <v>90.2</v>
       </c>
       <c r="AC13" t="s">
         <v>180</v>
@@ -3600,7 +3594,7 @@
         <v>183</v>
       </c>
       <c r="AQ13">
-        <v>8.4</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="AR13">
         <v>0</v>
@@ -3624,7 +3618,7 @@
         <v>199</v>
       </c>
       <c r="AY13">
-        <v>31.7</v>
+        <v>38.3</v>
       </c>
       <c r="AZ13">
         <v>5</v>
@@ -3755,7 +3749,7 @@
         <v>183</v>
       </c>
       <c r="AQ14">
-        <v>18.8</v>
+        <v>18.9</v>
       </c>
       <c r="AR14">
         <v>0</v>
@@ -3776,10 +3770,10 @@
         <v>7.1</v>
       </c>
       <c r="AX14" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="AY14">
-        <v>437.2</v>
+        <v>443.7</v>
       </c>
       <c r="AZ14">
         <v>5</v>
@@ -3910,7 +3904,7 @@
         <v>183</v>
       </c>
       <c r="AQ15">
-        <v>18.1</v>
+        <v>4.7</v>
       </c>
       <c r="AR15">
         <v>0</v>
@@ -3931,10 +3925,10 @@
         <v>22.2</v>
       </c>
       <c r="AX15" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="AY15">
-        <v>324.7</v>
+        <v>331.3</v>
       </c>
       <c r="AZ15">
         <v>5</v>
@@ -4065,7 +4059,7 @@
         <v>184</v>
       </c>
       <c r="AQ16">
-        <v>1.8</v>
+        <v>1.9</v>
       </c>
       <c r="AR16">
         <v>0</v>
@@ -4086,10 +4080,10 @@
         <v>18.1</v>
       </c>
       <c r="AX16" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="AY16">
-        <v>442.9</v>
+        <v>449.4</v>
       </c>
       <c r="AZ16">
         <v>5</v>
@@ -4211,211 +4205,211 @@
         <v>6</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>203</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>204</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>205</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>49</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>50</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="L1" s="1" t="s">
         <v>51</v>
       </c>
       <c r="M1" s="1" t="s">
+        <v>207</v>
+      </c>
+      <c r="N1" s="1" t="s">
         <v>208</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>209</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>210</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>212</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>213</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>214</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="U1" s="1" t="s">
         <v>215</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="V1" s="1" t="s">
         <v>216</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="W1" s="1" t="s">
         <v>217</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="X1" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>219</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>220</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>221</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AB1" s="1" t="s">
         <v>222</v>
       </c>
-      <c r="AB1" s="1" t="s">
+      <c r="AC1" s="1" t="s">
         <v>223</v>
       </c>
-      <c r="AC1" s="1" t="s">
+      <c r="AD1" s="1" t="s">
         <v>224</v>
       </c>
-      <c r="AD1" s="1" t="s">
+      <c r="AE1" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AE1" s="1" t="s">
+      <c r="AF1" s="1" t="s">
         <v>226</v>
       </c>
-      <c r="AF1" s="1" t="s">
+      <c r="AG1" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="AG1" s="1" t="s">
+      <c r="AH1" s="1" t="s">
         <v>228</v>
       </c>
-      <c r="AH1" s="1" t="s">
+      <c r="AI1" s="1" t="s">
         <v>229</v>
       </c>
-      <c r="AI1" s="1" t="s">
+      <c r="AJ1" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="AJ1" s="1" t="s">
+      <c r="AK1" s="1" t="s">
         <v>231</v>
       </c>
-      <c r="AK1" s="1" t="s">
+      <c r="AL1" s="1" t="s">
         <v>232</v>
       </c>
-      <c r="AL1" s="1" t="s">
+      <c r="AM1" s="1" t="s">
         <v>233</v>
       </c>
-      <c r="AM1" s="1" t="s">
+      <c r="AN1" s="1" t="s">
         <v>234</v>
       </c>
-      <c r="AN1" s="1" t="s">
+      <c r="AO1" s="1" t="s">
         <v>235</v>
       </c>
-      <c r="AO1" s="1" t="s">
+      <c r="AP1" s="1" t="s">
         <v>236</v>
       </c>
-      <c r="AP1" s="1" t="s">
+      <c r="AQ1" s="1" t="s">
         <v>237</v>
       </c>
-      <c r="AQ1" s="1" t="s">
+      <c r="AR1" s="1" t="s">
         <v>238</v>
       </c>
-      <c r="AR1" s="1" t="s">
+      <c r="AS1" s="1" t="s">
         <v>239</v>
       </c>
-      <c r="AS1" s="1" t="s">
+      <c r="AT1" s="1" t="s">
         <v>240</v>
       </c>
-      <c r="AT1" s="1" t="s">
+      <c r="AU1" s="1" t="s">
         <v>241</v>
       </c>
-      <c r="AU1" s="1" t="s">
+      <c r="AV1" s="1" t="s">
         <v>242</v>
       </c>
-      <c r="AV1" s="1" t="s">
+      <c r="AW1" s="1" t="s">
         <v>243</v>
       </c>
-      <c r="AW1" s="1" t="s">
+      <c r="AX1" s="1" t="s">
         <v>244</v>
       </c>
-      <c r="AX1" s="1" t="s">
+      <c r="AY1" s="1" t="s">
         <v>245</v>
       </c>
-      <c r="AY1" s="1" t="s">
+      <c r="AZ1" s="1" t="s">
         <v>246</v>
       </c>
-      <c r="AZ1" s="1" t="s">
+      <c r="BA1" s="1" t="s">
         <v>247</v>
       </c>
-      <c r="BA1" s="1" t="s">
+      <c r="BB1" s="1" t="s">
         <v>248</v>
       </c>
-      <c r="BB1" s="1" t="s">
+      <c r="BC1" s="1" t="s">
         <v>249</v>
       </c>
-      <c r="BC1" s="1" t="s">
+      <c r="BD1" s="1" t="s">
         <v>250</v>
       </c>
-      <c r="BD1" s="1" t="s">
+      <c r="BE1" s="1" t="s">
         <v>251</v>
       </c>
-      <c r="BE1" s="1" t="s">
+      <c r="BF1" s="1" t="s">
         <v>252</v>
       </c>
-      <c r="BF1" s="1" t="s">
+      <c r="BG1" s="1" t="s">
         <v>253</v>
       </c>
-      <c r="BG1" s="1" t="s">
+      <c r="BH1" s="1" t="s">
         <v>254</v>
       </c>
-      <c r="BH1" s="1" t="s">
+      <c r="BI1" s="1" t="s">
         <v>255</v>
       </c>
-      <c r="BI1" s="1" t="s">
+      <c r="BJ1" s="1" t="s">
         <v>256</v>
       </c>
-      <c r="BJ1" s="1" t="s">
+      <c r="BK1" s="1" t="s">
         <v>257</v>
       </c>
-      <c r="BK1" s="1" t="s">
+      <c r="BL1" s="1" t="s">
         <v>258</v>
       </c>
-      <c r="BL1" s="1" t="s">
+      <c r="BM1" s="1" t="s">
         <v>259</v>
       </c>
-      <c r="BM1" s="1" t="s">
+      <c r="BN1" s="1" t="s">
         <v>260</v>
       </c>
-      <c r="BN1" s="1" t="s">
+      <c r="BO1" s="1" t="s">
         <v>261</v>
       </c>
-      <c r="BO1" s="1" t="s">
+      <c r="BP1" s="1" t="s">
         <v>262</v>
       </c>
-      <c r="BP1" s="1" t="s">
+      <c r="BQ1" s="1" t="s">
         <v>263</v>
       </c>
-      <c r="BQ1" s="1" t="s">
+      <c r="BR1" s="1" t="s">
         <v>264</v>
       </c>
-      <c r="BR1" s="1" t="s">
+      <c r="BS1" s="1" t="s">
         <v>265</v>
       </c>
-      <c r="BS1" s="1" t="s">
+      <c r="BT1" s="1" t="s">
         <v>266</v>
       </c>
-      <c r="BT1" s="1" t="s">
+      <c r="BU1" s="1" t="s">
         <v>267</v>
-      </c>
-      <c r="BU1" s="1" t="s">
-        <v>268</v>
       </c>
       <c r="BV1" s="1" t="s">
         <v>48</v>
@@ -4424,16 +4418,16 @@
         <v>47</v>
       </c>
       <c r="BX1" s="1" t="s">
+        <v>268</v>
+      </c>
+      <c r="BY1" s="1" t="s">
         <v>269</v>
       </c>
-      <c r="BY1" s="1" t="s">
+      <c r="BZ1" s="1" t="s">
         <v>270</v>
       </c>
-      <c r="BZ1" s="1" t="s">
+      <c r="CA1" s="1" t="s">
         <v>271</v>
-      </c>
-      <c r="CA1" s="1" t="s">
-        <v>272</v>
       </c>
     </row>
     <row r="2" spans="1:79">
@@ -4450,25 +4444,25 @@
         <v>118</v>
       </c>
       <c r="E2" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F2" t="s">
         <v>106</v>
       </c>
       <c r="G2" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="H2" t="s">
         <v>188</v>
       </c>
       <c r="I2" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="J2">
-        <v>556</v>
+        <v>562.6</v>
       </c>
       <c r="K2">
-        <v>13.3</v>
+        <v>13.2</v>
       </c>
       <c r="L2">
         <v>5</v>
@@ -4495,13 +4489,13 @@
         <v>0</v>
       </c>
       <c r="T2" t="s">
+        <v>339</v>
+      </c>
+      <c r="U2" t="s">
+        <v>340</v>
+      </c>
+      <c r="V2" t="s">
         <v>341</v>
-      </c>
-      <c r="U2" t="s">
-        <v>342</v>
-      </c>
-      <c r="V2" t="s">
-        <v>343</v>
       </c>
       <c r="W2">
         <v>0.5833</v>
@@ -4618,7 +4612,7 @@
         <v>1.1658</v>
       </c>
       <c r="BI2" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="BJ2">
         <v>1595</v>
@@ -4689,25 +4683,25 @@
         <v>118</v>
       </c>
       <c r="E3" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="F3" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="G3" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="H3" t="s">
         <v>188</v>
       </c>
       <c r="I3" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="J3">
-        <v>556</v>
+        <v>562.6</v>
       </c>
       <c r="K3">
-        <v>14.3</v>
+        <v>14.2</v>
       </c>
       <c r="L3">
         <v>5</v>
@@ -4734,13 +4728,13 @@
         <v>0</v>
       </c>
       <c r="T3" t="s">
+        <v>339</v>
+      </c>
+      <c r="U3" t="s">
         <v>341</v>
       </c>
-      <c r="U3" t="s">
-        <v>343</v>
-      </c>
       <c r="V3" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="W3">
         <v>0.5833</v>
@@ -4767,7 +4761,7 @@
         <v>0.6</v>
       </c>
       <c r="AE3" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="AF3">
         <v>84.5</v>
@@ -4857,7 +4851,7 @@
         <v>1.1623</v>
       </c>
       <c r="BI3" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="BJ3">
         <v>1703</v>
@@ -4928,25 +4922,25 @@
         <v>118</v>
       </c>
       <c r="E4" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="F4" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="G4" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="H4" t="s">
         <v>188</v>
       </c>
       <c r="I4" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="J4">
-        <v>556</v>
+        <v>562.6</v>
       </c>
       <c r="K4">
-        <v>15.3</v>
+        <v>15.2</v>
       </c>
       <c r="L4">
         <v>5</v>
@@ -4973,13 +4967,13 @@
         <v>0</v>
       </c>
       <c r="T4" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="U4" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="V4" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="W4">
         <v>0.5833</v>
@@ -5096,7 +5090,7 @@
         <v>1.1606</v>
       </c>
       <c r="BI4" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="BJ4">
         <v>1761</v>
@@ -5167,25 +5161,25 @@
         <v>118</v>
       </c>
       <c r="E5" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="F5" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="G5" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="H5" t="s">
         <v>188</v>
       </c>
       <c r="I5" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="J5">
-        <v>556</v>
+        <v>562.6</v>
       </c>
       <c r="K5">
-        <v>16.3</v>
+        <v>16.2</v>
       </c>
       <c r="L5">
         <v>5</v>
@@ -5212,13 +5206,13 @@
         <v>0</v>
       </c>
       <c r="T5" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="U5" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="V5" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="W5">
         <v>0.5833</v>
@@ -5335,7 +5329,7 @@
         <v>1.1603</v>
       </c>
       <c r="BI5" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="BJ5">
         <v>1772</v>
@@ -5406,25 +5400,25 @@
         <v>119</v>
       </c>
       <c r="E6" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F6" t="s">
         <v>107</v>
       </c>
       <c r="G6" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="H6" t="s">
         <v>189</v>
       </c>
       <c r="I6" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="J6">
-        <v>336.4</v>
+        <v>343</v>
       </c>
       <c r="K6">
-        <v>18.8</v>
+        <v>18.7</v>
       </c>
       <c r="L6">
         <v>5</v>
@@ -5451,13 +5445,13 @@
         <v>0</v>
       </c>
       <c r="T6" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="U6" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="V6" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="W6">
         <v>0.0833</v>
@@ -5574,7 +5568,7 @@
         <v>1.156</v>
       </c>
       <c r="BI6" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="BJ6">
         <v>1880</v>
@@ -5645,25 +5639,25 @@
         <v>119</v>
       </c>
       <c r="E7" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="F7" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="G7" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="H7" t="s">
         <v>189</v>
       </c>
       <c r="I7" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="J7">
-        <v>336.4</v>
+        <v>343</v>
       </c>
       <c r="K7">
-        <v>19.8</v>
+        <v>19.7</v>
       </c>
       <c r="L7">
         <v>5</v>
@@ -5690,13 +5684,13 @@
         <v>56.2</v>
       </c>
       <c r="T7" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="U7" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="V7" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="W7">
         <v>0.0833</v>
@@ -5765,7 +5759,7 @@
         <v>7</v>
       </c>
       <c r="AS7" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="AT7">
         <v>75.59999999999999</v>
@@ -5813,7 +5807,7 @@
         <v>1.1612</v>
       </c>
       <c r="BI7" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="BJ7">
         <v>1705</v>
@@ -5884,25 +5878,25 @@
         <v>119</v>
       </c>
       <c r="E8" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="F8" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="G8" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="H8" t="s">
         <v>189</v>
       </c>
       <c r="I8" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="J8">
-        <v>336.4</v>
+        <v>343</v>
       </c>
       <c r="K8">
-        <v>20.8</v>
+        <v>20.7</v>
       </c>
       <c r="L8">
         <v>5</v>
@@ -5929,13 +5923,13 @@
         <v>75</v>
       </c>
       <c r="T8" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="U8" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="V8" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="W8">
         <v>0.0833</v>
@@ -6052,7 +6046,7 @@
         <v>1.169</v>
       </c>
       <c r="BI8" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="BJ8">
         <v>1415</v>
@@ -6091,7 +6085,7 @@
         <v>185</v>
       </c>
       <c r="BV8">
-        <v>4.8</v>
+        <v>4.7</v>
       </c>
       <c r="BW8" t="s">
         <v>185</v>
@@ -6123,25 +6117,25 @@
         <v>119</v>
       </c>
       <c r="E9" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="F9" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="G9" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="H9" t="s">
         <v>189</v>
       </c>
       <c r="I9" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="J9">
-        <v>336.4</v>
+        <v>343</v>
       </c>
       <c r="K9">
-        <v>21.8</v>
+        <v>21.7</v>
       </c>
       <c r="L9">
         <v>5</v>
@@ -6168,13 +6162,13 @@
         <v>100</v>
       </c>
       <c r="T9" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="U9" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="V9" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="W9">
         <v>0.0833</v>
@@ -6243,7 +6237,7 @@
         <v>9.4</v>
       </c>
       <c r="AS9" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="AT9">
         <v>150.3</v>
@@ -6291,7 +6285,7 @@
         <v>1.1726</v>
       </c>
       <c r="BI9" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="BJ9">
         <v>1288</v>
@@ -6362,25 +6356,25 @@
         <v>118</v>
       </c>
       <c r="E10" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F10" t="s">
         <v>108</v>
       </c>
       <c r="G10" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="H10" t="s">
         <v>190</v>
       </c>
       <c r="I10" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="J10">
-        <v>556</v>
+        <v>562.7</v>
       </c>
       <c r="K10">
-        <v>18.9</v>
+        <v>18.8</v>
       </c>
       <c r="L10">
         <v>5</v>
@@ -6407,13 +6401,13 @@
         <v>25</v>
       </c>
       <c r="T10" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="U10" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="V10" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="W10">
         <v>0.1667</v>
@@ -6530,7 +6524,7 @@
         <v>1.1688</v>
       </c>
       <c r="BI10" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="BJ10">
         <v>1505</v>
@@ -6601,25 +6595,25 @@
         <v>118</v>
       </c>
       <c r="E11" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="F11" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="G11" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="H11" t="s">
         <v>190</v>
       </c>
       <c r="I11" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="J11">
-        <v>556</v>
+        <v>562.7</v>
       </c>
       <c r="K11">
-        <v>19.9</v>
+        <v>19.8</v>
       </c>
       <c r="L11">
         <v>5</v>
@@ -6646,13 +6640,13 @@
         <v>81.2</v>
       </c>
       <c r="T11" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="U11" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="V11" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="W11">
         <v>0.1667</v>
@@ -6721,7 +6715,7 @@
         <v>8.699999999999999</v>
       </c>
       <c r="AS11" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="AT11">
         <v>316.6</v>
@@ -6769,7 +6763,7 @@
         <v>1.1761</v>
       </c>
       <c r="BI11" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="BJ11">
         <v>1275</v>
@@ -6840,25 +6834,25 @@
         <v>118</v>
       </c>
       <c r="E12" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="F12" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="G12" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="H12" t="s">
         <v>190</v>
       </c>
       <c r="I12" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="J12">
-        <v>556</v>
+        <v>562.7</v>
       </c>
       <c r="K12">
-        <v>20.9</v>
+        <v>20.8</v>
       </c>
       <c r="L12">
         <v>5</v>
@@ -6885,13 +6879,13 @@
         <v>81.2</v>
       </c>
       <c r="T12" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="U12" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="V12" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="W12">
         <v>0.1667</v>
@@ -6918,7 +6912,7 @@
         <v>0.6</v>
       </c>
       <c r="AE12" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="AF12">
         <v>74.90000000000001</v>
@@ -7008,7 +7002,7 @@
         <v>1.1831</v>
       </c>
       <c r="BI12" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="BJ12">
         <v>1049</v>
@@ -7079,25 +7073,25 @@
         <v>118</v>
       </c>
       <c r="E13" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="F13" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="G13" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="H13" t="s">
         <v>190</v>
       </c>
       <c r="I13" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="J13">
-        <v>556</v>
+        <v>562.7</v>
       </c>
       <c r="K13">
-        <v>21.9</v>
+        <v>21.8</v>
       </c>
       <c r="L13">
         <v>5</v>
@@ -7124,13 +7118,13 @@
         <v>81.2</v>
       </c>
       <c r="T13" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="U13" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="V13" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="W13">
         <v>0.1667</v>
@@ -7199,7 +7193,7 @@
         <v>7.2</v>
       </c>
       <c r="AS13" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="AT13">
         <v>144.5</v>
@@ -7247,7 +7241,7 @@
         <v>1.189</v>
       </c>
       <c r="BI13" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="BJ13">
         <v>873</v>
@@ -7318,25 +7312,25 @@
         <v>120</v>
       </c>
       <c r="E14" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F14" t="s">
         <v>108</v>
       </c>
       <c r="G14" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="H14" t="s">
         <v>191</v>
       </c>
       <c r="I14" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="J14">
-        <v>481.2</v>
+        <v>487.8</v>
       </c>
       <c r="K14">
-        <v>18.9</v>
+        <v>18.8</v>
       </c>
       <c r="L14">
         <v>5</v>
@@ -7363,13 +7357,13 @@
         <v>56.2</v>
       </c>
       <c r="T14" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="U14" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="V14" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="W14">
         <v>0.1667</v>
@@ -7486,7 +7480,7 @@
         <v>1.1393</v>
       </c>
       <c r="BI14" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="BJ14">
         <v>2273</v>
@@ -7525,7 +7519,7 @@
         <v>185</v>
       </c>
       <c r="BV14">
-        <v>3.1</v>
+        <v>3</v>
       </c>
       <c r="BW14" t="s">
         <v>185</v>
@@ -7557,25 +7551,25 @@
         <v>120</v>
       </c>
       <c r="E15" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="F15" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="G15" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="H15" t="s">
         <v>191</v>
       </c>
       <c r="I15" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="J15">
-        <v>481.2</v>
+        <v>487.8</v>
       </c>
       <c r="K15">
-        <v>19.9</v>
+        <v>19.8</v>
       </c>
       <c r="L15">
         <v>5</v>
@@ -7602,13 +7596,13 @@
         <v>56.2</v>
       </c>
       <c r="T15" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="U15" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="V15" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="W15">
         <v>0.1667</v>
@@ -7617,7 +7611,7 @@
         <v>6.5</v>
       </c>
       <c r="Y15">
-        <v>93.7</v>
+        <v>93.8</v>
       </c>
       <c r="Z15">
         <v>63.4</v>
@@ -7677,7 +7671,7 @@
         <v>5.8</v>
       </c>
       <c r="AS15" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="AT15">
         <v>78.2</v>
@@ -7725,7 +7719,7 @@
         <v>1.1418</v>
       </c>
       <c r="BI15" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="BJ15">
         <v>2187</v>
@@ -7796,25 +7790,25 @@
         <v>120</v>
       </c>
       <c r="E16" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="F16" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="G16" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="H16" t="s">
         <v>191</v>
       </c>
       <c r="I16" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="J16">
-        <v>481.2</v>
+        <v>487.8</v>
       </c>
       <c r="K16">
-        <v>20.9</v>
+        <v>20.8</v>
       </c>
       <c r="L16">
         <v>5</v>
@@ -7841,13 +7835,13 @@
         <v>56.2</v>
       </c>
       <c r="T16" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="U16" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="V16" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="W16">
         <v>0.1667</v>
@@ -7916,7 +7910,7 @@
         <v>6</v>
       </c>
       <c r="AS16" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="AT16">
         <v>133.6</v>
@@ -7964,7 +7958,7 @@
         <v>1.1467</v>
       </c>
       <c r="BI16" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="BJ16">
         <v>2033</v>
@@ -8035,25 +8029,25 @@
         <v>120</v>
       </c>
       <c r="E17" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="F17" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="G17" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="H17" t="s">
         <v>191</v>
       </c>
       <c r="I17" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="J17">
-        <v>481.2</v>
+        <v>487.8</v>
       </c>
       <c r="K17">
-        <v>21.9</v>
+        <v>21.8</v>
       </c>
       <c r="L17">
         <v>5</v>
@@ -8080,13 +8074,13 @@
         <v>0</v>
       </c>
       <c r="T17" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="U17" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="V17" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="W17">
         <v>0.1667</v>
@@ -8095,7 +8089,7 @@
         <v>8.5</v>
       </c>
       <c r="Y17">
-        <v>89.59999999999999</v>
+        <v>89.7</v>
       </c>
       <c r="Z17">
         <v>67.5</v>
@@ -8203,7 +8197,7 @@
         <v>1.1488</v>
       </c>
       <c r="BI17" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="BJ17">
         <v>1977</v>
@@ -8274,25 +8268,25 @@
         <v>121</v>
       </c>
       <c r="E18" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F18" t="s">
         <v>109</v>
       </c>
       <c r="G18" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="H18" t="s">
         <v>192</v>
       </c>
       <c r="I18" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="J18">
-        <v>325.3</v>
+        <v>331.9</v>
       </c>
       <c r="K18">
-        <v>19</v>
+        <v>18.8</v>
       </c>
       <c r="L18">
         <v>5</v>
@@ -8319,13 +8313,13 @@
         <v>0</v>
       </c>
       <c r="T18" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="U18" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="V18" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="W18">
         <v>0.25</v>
@@ -8442,7 +8436,7 @@
         <v>1.123</v>
       </c>
       <c r="BI18" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="BJ18">
         <v>2642</v>
@@ -8513,25 +8507,25 @@
         <v>121</v>
       </c>
       <c r="E19" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="F19" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="G19" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="H19" t="s">
         <v>192</v>
       </c>
       <c r="I19" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="J19">
-        <v>325.3</v>
+        <v>331.9</v>
       </c>
       <c r="K19">
-        <v>20</v>
+        <v>19.8</v>
       </c>
       <c r="L19">
         <v>5</v>
@@ -8558,13 +8552,13 @@
         <v>0</v>
       </c>
       <c r="T19" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="U19" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="V19" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="W19">
         <v>0.25</v>
@@ -8681,7 +8675,7 @@
         <v>1.1261</v>
       </c>
       <c r="BI19" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="BJ19">
         <v>2547</v>
@@ -8720,7 +8714,7 @@
         <v>186</v>
       </c>
       <c r="BV19">
-        <v>2.9</v>
+        <v>2.8</v>
       </c>
       <c r="BW19" t="s">
         <v>185</v>
@@ -8752,25 +8746,25 @@
         <v>121</v>
       </c>
       <c r="E20" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="F20" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="G20" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="H20" t="s">
         <v>192</v>
       </c>
       <c r="I20" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="J20">
-        <v>325.3</v>
+        <v>331.9</v>
       </c>
       <c r="K20">
-        <v>21</v>
+        <v>20.8</v>
       </c>
       <c r="L20">
         <v>5</v>
@@ -8797,13 +8791,13 @@
         <v>0</v>
       </c>
       <c r="T20" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="U20" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="V20" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="W20">
         <v>0.25</v>
@@ -8872,7 +8866,7 @@
         <v>14.4</v>
       </c>
       <c r="AS20" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="AT20">
         <v>305.7</v>
@@ -8920,7 +8914,7 @@
         <v>1.1303</v>
       </c>
       <c r="BI20" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="BJ20">
         <v>2417</v>
@@ -8991,25 +8985,25 @@
         <v>121</v>
       </c>
       <c r="E21" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="F21" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="G21" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="H21" t="s">
         <v>192</v>
       </c>
       <c r="I21" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="J21">
-        <v>325.3</v>
+        <v>331.9</v>
       </c>
       <c r="K21">
-        <v>22</v>
+        <v>21.8</v>
       </c>
       <c r="L21">
         <v>5</v>
@@ -9036,13 +9030,13 @@
         <v>0</v>
       </c>
       <c r="T21" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="U21" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="V21" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="W21">
         <v>0.25</v>
@@ -9111,7 +9105,7 @@
         <v>12.1</v>
       </c>
       <c r="AS21" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="AT21">
         <v>307.5</v>
@@ -9159,7 +9153,7 @@
         <v>1.1347</v>
       </c>
       <c r="BI21" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="BJ21">
         <v>2283</v>
@@ -9230,13 +9224,13 @@
         <v>122</v>
       </c>
       <c r="E22" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F22" t="s">
         <v>109</v>
       </c>
       <c r="G22" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="H22" t="s">
         <v>193</v>
@@ -9245,7 +9239,7 @@
         <v>0</v>
       </c>
       <c r="K22">
-        <v>19</v>
+        <v>18.8</v>
       </c>
       <c r="L22">
         <v>4</v>
@@ -9272,13 +9266,13 @@
         <v>0</v>
       </c>
       <c r="T22" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="U22" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="V22" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="W22">
         <v>0.25</v>
@@ -9395,7 +9389,7 @@
         <v>1.171</v>
       </c>
       <c r="BI22" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="BJ22">
         <v>1338</v>
@@ -9463,13 +9457,13 @@
         <v>122</v>
       </c>
       <c r="E23" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="F23" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="G23" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="H23" t="s">
         <v>193</v>
@@ -9478,7 +9472,7 @@
         <v>0</v>
       </c>
       <c r="K23">
-        <v>20</v>
+        <v>19.8</v>
       </c>
       <c r="L23">
         <v>4</v>
@@ -9505,13 +9499,13 @@
         <v>56.2</v>
       </c>
       <c r="T23" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="U23" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="V23" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="W23">
         <v>0.25</v>
@@ -9538,7 +9532,7 @@
         <v>0.2</v>
       </c>
       <c r="AE23" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="AF23">
         <v>73.8</v>
@@ -9628,7 +9622,7 @@
         <v>1.1724</v>
       </c>
       <c r="BI23" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="BJ23">
         <v>1295</v>
@@ -9696,13 +9690,13 @@
         <v>122</v>
       </c>
       <c r="E24" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="F24" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="G24" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="H24" t="s">
         <v>193</v>
@@ -9711,7 +9705,7 @@
         <v>0</v>
       </c>
       <c r="K24">
-        <v>21</v>
+        <v>20.8</v>
       </c>
       <c r="L24">
         <v>4</v>
@@ -9738,13 +9732,13 @@
         <v>56.2</v>
       </c>
       <c r="T24" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="U24" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="V24" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="W24">
         <v>0.25</v>
@@ -9861,7 +9855,7 @@
         <v>1.1749</v>
       </c>
       <c r="BI24" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="BJ24">
         <v>1218</v>
@@ -9929,13 +9923,13 @@
         <v>122</v>
       </c>
       <c r="E25" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="F25" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="G25" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="H25" t="s">
         <v>193</v>
@@ -9944,7 +9938,7 @@
         <v>0</v>
       </c>
       <c r="K25">
-        <v>22</v>
+        <v>21.8</v>
       </c>
       <c r="L25">
         <v>4</v>
@@ -9971,13 +9965,13 @@
         <v>56.2</v>
       </c>
       <c r="T25" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="U25" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="V25" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="W25">
         <v>0.25</v>
@@ -10046,7 +10040,7 @@
         <v>5.7</v>
       </c>
       <c r="AS25" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="AT25">
         <v>76.8</v>
@@ -10094,7 +10088,7 @@
         <v>1.1748</v>
       </c>
       <c r="BI25" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="BJ25">
         <v>1226</v>
@@ -10162,25 +10156,25 @@
         <v>123</v>
       </c>
       <c r="E26" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F26" t="s">
         <v>110</v>
       </c>
       <c r="G26" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="H26" t="s">
         <v>194</v>
       </c>
       <c r="I26" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="J26">
-        <v>160.7</v>
+        <v>167.3</v>
       </c>
       <c r="K26">
-        <v>19.4</v>
+        <v>19.3</v>
       </c>
       <c r="L26">
         <v>5</v>
@@ -10207,13 +10201,13 @@
         <v>100</v>
       </c>
       <c r="T26" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="U26" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="V26" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="W26">
         <v>0.6667</v>
@@ -10330,7 +10324,7 @@
         <v>1.1896</v>
       </c>
       <c r="BI26" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="BJ26">
         <v>858</v>
@@ -10366,7 +10360,7 @@
         <v>0</v>
       </c>
       <c r="BU26" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="BV26">
         <v>9.6</v>
@@ -10401,25 +10395,25 @@
         <v>123</v>
       </c>
       <c r="E27" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="F27" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="G27" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="H27" t="s">
         <v>194</v>
       </c>
       <c r="I27" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="J27">
-        <v>160.7</v>
+        <v>167.3</v>
       </c>
       <c r="K27">
-        <v>20.4</v>
+        <v>20.3</v>
       </c>
       <c r="L27">
         <v>5</v>
@@ -10446,13 +10440,13 @@
         <v>100</v>
       </c>
       <c r="T27" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="U27" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="V27" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="W27">
         <v>0.6667</v>
@@ -10479,7 +10473,7 @@
         <v>0.5</v>
       </c>
       <c r="AE27" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="AF27">
         <v>84.59999999999999</v>
@@ -10569,7 +10563,7 @@
         <v>1.1268</v>
       </c>
       <c r="BI27" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="BJ27">
         <v>2568</v>
@@ -10640,25 +10634,25 @@
         <v>123</v>
       </c>
       <c r="E28" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="F28" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="G28" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="H28" t="s">
         <v>194</v>
       </c>
       <c r="I28" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="J28">
-        <v>160.7</v>
+        <v>167.3</v>
       </c>
       <c r="K28">
-        <v>21.4</v>
+        <v>21.3</v>
       </c>
       <c r="L28">
         <v>5</v>
@@ -10685,13 +10679,13 @@
         <v>0</v>
       </c>
       <c r="T28" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="U28" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="V28" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="W28">
         <v>0.6667</v>
@@ -10718,7 +10712,7 @@
         <v>0.5</v>
       </c>
       <c r="AE28" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="AF28">
         <v>82.40000000000001</v>
@@ -10808,7 +10802,7 @@
         <v>1.1311</v>
       </c>
       <c r="BI28" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="BJ28">
         <v>2428</v>
@@ -10879,25 +10873,25 @@
         <v>123</v>
       </c>
       <c r="E29" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="F29" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="G29" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="H29" t="s">
         <v>194</v>
       </c>
       <c r="I29" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="J29">
-        <v>160.7</v>
+        <v>167.3</v>
       </c>
       <c r="K29">
-        <v>22.4</v>
+        <v>22.3</v>
       </c>
       <c r="L29">
         <v>5</v>
@@ -10924,13 +10918,13 @@
         <v>0</v>
       </c>
       <c r="T29" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="U29" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="V29" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="W29">
         <v>0.6667</v>
@@ -11047,7 +11041,7 @@
         <v>1.1348</v>
       </c>
       <c r="BI29" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="BJ29">
         <v>2316</v>
@@ -11118,25 +11112,25 @@
         <v>124</v>
       </c>
       <c r="E30" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F30" t="s">
         <v>111</v>
       </c>
       <c r="G30" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H30" t="s">
         <v>195</v>
       </c>
       <c r="I30" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="J30">
-        <v>56.6</v>
+        <v>63.2</v>
       </c>
       <c r="K30">
-        <v>19.8</v>
+        <v>19.7</v>
       </c>
       <c r="L30">
         <v>5</v>
@@ -11163,13 +11157,13 @@
         <v>0</v>
       </c>
       <c r="T30" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="U30" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="V30" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="W30">
         <v>0.0833</v>
@@ -11286,7 +11280,7 @@
         <v>1.1497</v>
       </c>
       <c r="BI30" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="BJ30">
         <v>1889</v>
@@ -11357,25 +11351,25 @@
         <v>124</v>
       </c>
       <c r="E31" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="F31" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="G31" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H31" t="s">
         <v>195</v>
       </c>
       <c r="I31" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="J31">
-        <v>56.6</v>
+        <v>63.2</v>
       </c>
       <c r="K31">
-        <v>20.8</v>
+        <v>20.7</v>
       </c>
       <c r="L31">
         <v>5</v>
@@ -11402,13 +11396,13 @@
         <v>0</v>
       </c>
       <c r="T31" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="U31" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="V31" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="W31">
         <v>0.0833</v>
@@ -11525,7 +11519,7 @@
         <v>1.1518</v>
       </c>
       <c r="BI31" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="BJ31">
         <v>1821</v>
@@ -11596,25 +11590,25 @@
         <v>124</v>
       </c>
       <c r="E32" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="F32" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="G32" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H32" t="s">
         <v>195</v>
       </c>
       <c r="I32" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="J32">
-        <v>56.6</v>
+        <v>63.2</v>
       </c>
       <c r="K32">
-        <v>21.8</v>
+        <v>21.7</v>
       </c>
       <c r="L32">
         <v>5</v>
@@ -11641,13 +11635,13 @@
         <v>0</v>
       </c>
       <c r="T32" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="U32" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="V32" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="W32">
         <v>0.0833</v>
@@ -11764,7 +11758,7 @@
         <v>1.1537</v>
       </c>
       <c r="BI32" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="BJ32">
         <v>1747</v>
@@ -11835,25 +11829,25 @@
         <v>124</v>
       </c>
       <c r="E33" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="F33" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="G33" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H33" t="s">
         <v>195</v>
       </c>
       <c r="I33" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="J33">
-        <v>56.6</v>
+        <v>63.2</v>
       </c>
       <c r="K33">
-        <v>22.8</v>
+        <v>22.7</v>
       </c>
       <c r="L33">
         <v>5</v>
@@ -11880,13 +11874,13 @@
         <v>0</v>
       </c>
       <c r="T33" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="U33" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="V33" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="W33">
         <v>0.0833</v>
@@ -11913,7 +11907,7 @@
         <v>1.8</v>
       </c>
       <c r="AE33" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="AF33">
         <v>81.09999999999999</v>
@@ -12003,7 +11997,7 @@
         <v>1.1564</v>
       </c>
       <c r="BI33" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="BJ33">
         <v>1654</v>
@@ -12074,25 +12068,25 @@
         <v>125</v>
       </c>
       <c r="E34" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F34" t="s">
         <v>112</v>
       </c>
       <c r="G34" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="H34" t="s">
         <v>196</v>
       </c>
       <c r="I34" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="J34">
-        <v>31.6</v>
+        <v>38.2</v>
       </c>
       <c r="K34">
-        <v>19.9</v>
+        <v>19.8</v>
       </c>
       <c r="L34">
         <v>5</v>
@@ -12119,13 +12113,13 @@
         <v>0</v>
       </c>
       <c r="T34" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="U34" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="V34" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="W34">
         <v>0.1667</v>
@@ -12242,7 +12236,7 @@
         <v>1.1896</v>
       </c>
       <c r="BI34" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="BJ34">
         <v>858</v>
@@ -12278,7 +12272,7 @@
         <v>0</v>
       </c>
       <c r="BU34" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="BV34">
         <v>13</v>
@@ -12313,25 +12307,25 @@
         <v>125</v>
       </c>
       <c r="E35" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="F35" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="G35" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="H35" t="s">
         <v>196</v>
       </c>
       <c r="I35" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="J35">
-        <v>31.6</v>
+        <v>38.2</v>
       </c>
       <c r="K35">
-        <v>20.9</v>
+        <v>20.8</v>
       </c>
       <c r="L35">
         <v>5</v>
@@ -12358,13 +12352,13 @@
         <v>0</v>
       </c>
       <c r="T35" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="U35" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="V35" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="W35">
         <v>0.1667</v>
@@ -12373,7 +12367,7 @@
         <v>12.1</v>
       </c>
       <c r="Y35">
-        <v>85.8</v>
+        <v>85.90000000000001</v>
       </c>
       <c r="Z35">
         <v>71.5</v>
@@ -12481,7 +12475,7 @@
         <v>1.1575</v>
       </c>
       <c r="BI35" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="BJ35">
         <v>1621</v>
@@ -12552,25 +12546,25 @@
         <v>125</v>
       </c>
       <c r="E36" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="F36" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="G36" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="H36" t="s">
         <v>196</v>
       </c>
       <c r="I36" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="J36">
-        <v>31.6</v>
+        <v>38.2</v>
       </c>
       <c r="K36">
-        <v>21.9</v>
+        <v>21.8</v>
       </c>
       <c r="L36">
         <v>5</v>
@@ -12597,13 +12591,13 @@
         <v>0</v>
       </c>
       <c r="T36" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="U36" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="V36" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="W36">
         <v>0.1667</v>
@@ -12720,7 +12714,7 @@
         <v>1.1622</v>
       </c>
       <c r="BI36" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="BJ36">
         <v>1467</v>
@@ -12791,25 +12785,25 @@
         <v>125</v>
       </c>
       <c r="E37" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="F37" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="G37" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="H37" t="s">
         <v>196</v>
       </c>
       <c r="I37" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="J37">
-        <v>31.6</v>
+        <v>38.2</v>
       </c>
       <c r="K37">
-        <v>22.9</v>
+        <v>22.8</v>
       </c>
       <c r="L37">
         <v>5</v>
@@ -12836,13 +12830,13 @@
         <v>0</v>
       </c>
       <c r="T37" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="U37" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="V37" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="W37">
         <v>0.1667</v>
@@ -12959,7 +12953,7 @@
         <v>1.1646</v>
       </c>
       <c r="BI37" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="BJ37">
         <v>1385</v>
@@ -13030,25 +13024,25 @@
         <v>126</v>
       </c>
       <c r="E38" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F38" t="s">
         <v>112</v>
       </c>
       <c r="G38" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="H38" t="s">
         <v>197</v>
       </c>
       <c r="I38" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="J38">
-        <v>5.9</v>
+        <v>12.4</v>
       </c>
       <c r="K38">
-        <v>19.9</v>
+        <v>19.8</v>
       </c>
       <c r="L38">
         <v>5</v>
@@ -13075,13 +13069,13 @@
         <v>0</v>
       </c>
       <c r="T38" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="U38" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="V38" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="W38">
         <v>0.1667</v>
@@ -13198,7 +13192,7 @@
         <v>1.1173</v>
       </c>
       <c r="BI38" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="BJ38">
         <v>2873</v>
@@ -13269,25 +13263,25 @@
         <v>126</v>
       </c>
       <c r="E39" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="F39" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="G39" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="H39" t="s">
         <v>197</v>
       </c>
       <c r="I39" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="J39">
-        <v>5.9</v>
+        <v>12.4</v>
       </c>
       <c r="K39">
-        <v>20.9</v>
+        <v>20.8</v>
       </c>
       <c r="L39">
         <v>5</v>
@@ -13314,13 +13308,13 @@
         <v>0</v>
       </c>
       <c r="T39" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="U39" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="V39" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="W39">
         <v>0.1667</v>
@@ -13437,7 +13431,7 @@
         <v>1.1216</v>
       </c>
       <c r="BI39" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="BJ39">
         <v>2731</v>
@@ -13508,25 +13502,25 @@
         <v>126</v>
       </c>
       <c r="E40" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="F40" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="G40" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="H40" t="s">
         <v>197</v>
       </c>
       <c r="I40" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="J40">
-        <v>5.9</v>
+        <v>12.4</v>
       </c>
       <c r="K40">
-        <v>21.9</v>
+        <v>21.8</v>
       </c>
       <c r="L40">
         <v>5</v>
@@ -13553,13 +13547,13 @@
         <v>0</v>
       </c>
       <c r="T40" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="U40" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="V40" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="W40">
         <v>0.1667</v>
@@ -13676,7 +13670,7 @@
         <v>1.1259</v>
       </c>
       <c r="BI40" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="BJ40">
         <v>2592</v>
@@ -13747,25 +13741,25 @@
         <v>126</v>
       </c>
       <c r="E41" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="F41" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="G41" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="H41" t="s">
         <v>197</v>
       </c>
       <c r="I41" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="J41">
-        <v>5.9</v>
+        <v>12.4</v>
       </c>
       <c r="K41">
-        <v>22.9</v>
+        <v>22.8</v>
       </c>
       <c r="L41">
         <v>5</v>
@@ -13792,13 +13786,13 @@
         <v>0</v>
       </c>
       <c r="T41" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="U41" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="V41" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="W41">
         <v>0.1667</v>
@@ -13915,7 +13909,7 @@
         <v>1.13</v>
       </c>
       <c r="BI41" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="BJ41">
         <v>2461</v>
@@ -13986,25 +13980,25 @@
         <v>127</v>
       </c>
       <c r="E42" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F42" t="s">
         <v>113</v>
       </c>
       <c r="G42" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="H42" t="s">
         <v>198</v>
       </c>
       <c r="I42" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="J42">
-        <v>571.6</v>
+        <v>578.2</v>
       </c>
       <c r="K42">
-        <v>20.4</v>
+        <v>20.3</v>
       </c>
       <c r="L42">
         <v>5</v>
@@ -14031,13 +14025,13 @@
         <v>75</v>
       </c>
       <c r="T42" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="U42" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="V42" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="W42">
         <v>0.6667</v>
@@ -14046,7 +14040,7 @@
         <v>11.5</v>
       </c>
       <c r="Y42">
-        <v>92.40000000000001</v>
+        <v>92.5</v>
       </c>
       <c r="Z42">
         <v>94.2</v>
@@ -14154,7 +14148,7 @@
         <v>0.9556</v>
       </c>
       <c r="BI42" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="BJ42">
         <v>8309</v>
@@ -14225,25 +14219,25 @@
         <v>127</v>
       </c>
       <c r="E43" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="F43" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="G43" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="H43" t="s">
         <v>198</v>
       </c>
       <c r="I43" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="J43">
-        <v>571.6</v>
+        <v>578.2</v>
       </c>
       <c r="K43">
-        <v>21.4</v>
+        <v>21.3</v>
       </c>
       <c r="L43">
         <v>5</v>
@@ -14270,13 +14264,13 @@
         <v>75</v>
       </c>
       <c r="T43" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="U43" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="V43" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="W43">
         <v>0.6667</v>
@@ -14393,7 +14387,7 @@
         <v>0.9583</v>
       </c>
       <c r="BI43" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="BJ43">
         <v>8204</v>
@@ -14464,25 +14458,25 @@
         <v>127</v>
       </c>
       <c r="E44" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="F44" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="G44" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="H44" t="s">
         <v>198</v>
       </c>
       <c r="I44" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="J44">
-        <v>571.6</v>
+        <v>578.2</v>
       </c>
       <c r="K44">
-        <v>22.4</v>
+        <v>22.3</v>
       </c>
       <c r="L44">
         <v>5</v>
@@ -14509,13 +14503,13 @@
         <v>0</v>
       </c>
       <c r="T44" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="U44" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="V44" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="W44">
         <v>0.6667</v>
@@ -14632,7 +14626,7 @@
         <v>0.9641999999999999</v>
       </c>
       <c r="BI44" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="BJ44">
         <v>7979</v>
@@ -14703,25 +14697,25 @@
         <v>127</v>
       </c>
       <c r="E45" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="F45" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="G45" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="H45" t="s">
         <v>198</v>
       </c>
       <c r="I45" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="J45">
-        <v>571.6</v>
+        <v>578.2</v>
       </c>
       <c r="K45">
-        <v>23.4</v>
+        <v>23.3</v>
       </c>
       <c r="L45">
         <v>5</v>
@@ -14748,13 +14742,13 @@
         <v>0</v>
       </c>
       <c r="T45" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="U45" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="V45" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="W45">
         <v>0.6667</v>
@@ -14781,7 +14775,7 @@
         <v>4</v>
       </c>
       <c r="AE45" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="AF45">
         <v>84.09999999999999</v>
@@ -14823,7 +14817,7 @@
         <v>19.4</v>
       </c>
       <c r="AS45" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="AT45">
         <v>132.2</v>
@@ -14871,7 +14865,7 @@
         <v>0.9697</v>
       </c>
       <c r="BI45" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="BJ45">
         <v>7772</v>
@@ -14942,25 +14936,25 @@
         <v>128</v>
       </c>
       <c r="E46" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F46" t="s">
         <v>114</v>
       </c>
       <c r="G46" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="H46" t="s">
         <v>199</v>
       </c>
       <c r="I46" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="J46">
-        <v>31.7</v>
+        <v>38.3</v>
       </c>
       <c r="K46">
-        <v>21.3</v>
+        <v>21.2</v>
       </c>
       <c r="L46">
         <v>5</v>
@@ -14987,13 +14981,13 @@
         <v>0</v>
       </c>
       <c r="T46" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="U46" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="V46" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="W46">
         <v>0.6333</v>
@@ -15110,7 +15104,7 @@
         <v>1.1717</v>
       </c>
       <c r="BI46" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="BJ46">
         <v>1281</v>
@@ -15181,25 +15175,25 @@
         <v>128</v>
       </c>
       <c r="E47" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="F47" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="G47" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="H47" t="s">
         <v>199</v>
       </c>
       <c r="I47" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="J47">
-        <v>31.7</v>
+        <v>38.3</v>
       </c>
       <c r="K47">
-        <v>22.3</v>
+        <v>22.2</v>
       </c>
       <c r="L47">
         <v>5</v>
@@ -15226,13 +15220,13 @@
         <v>0</v>
       </c>
       <c r="T47" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="U47" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="V47" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="W47">
         <v>0.6333</v>
@@ -15241,7 +15235,7 @@
         <v>6.5</v>
       </c>
       <c r="Y47">
-        <v>89.7</v>
+        <v>89.8</v>
       </c>
       <c r="Z47">
         <v>64.8</v>
@@ -15349,7 +15343,7 @@
         <v>1.1783</v>
       </c>
       <c r="BI47" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="BJ47">
         <v>1087</v>
@@ -15420,25 +15414,25 @@
         <v>128</v>
       </c>
       <c r="E48" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="F48" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="G48" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="H48" t="s">
         <v>199</v>
       </c>
       <c r="I48" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="J48">
-        <v>31.7</v>
+        <v>38.3</v>
       </c>
       <c r="K48">
-        <v>23.3</v>
+        <v>23.2</v>
       </c>
       <c r="L48">
         <v>5</v>
@@ -15465,13 +15459,13 @@
         <v>0</v>
       </c>
       <c r="T48" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="U48" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="V48" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="W48">
         <v>0.6333</v>
@@ -15498,7 +15492,7 @@
         <v>0</v>
       </c>
       <c r="AE48" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="AF48">
         <v>72.09999999999999</v>
@@ -15588,7 +15582,7 @@
         <v>1.1839</v>
       </c>
       <c r="BI48" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="BJ48">
         <v>917</v>
@@ -15659,25 +15653,25 @@
         <v>128</v>
       </c>
       <c r="E49" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="F49" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="G49" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="H49" t="s">
         <v>199</v>
       </c>
       <c r="I49" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="J49">
-        <v>31.7</v>
+        <v>38.3</v>
       </c>
       <c r="K49">
-        <v>24.3</v>
+        <v>24.2</v>
       </c>
       <c r="L49">
         <v>5</v>
@@ -15704,13 +15698,13 @@
         <v>0</v>
       </c>
       <c r="T49" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="U49" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="V49" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="W49">
         <v>0.6333</v>
@@ -15827,7 +15821,7 @@
         <v>1.1875</v>
       </c>
       <c r="BI49" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="BJ49">
         <v>808</v>
@@ -15898,25 +15892,25 @@
         <v>129</v>
       </c>
       <c r="E50" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F50" t="s">
         <v>115</v>
       </c>
       <c r="G50" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="H50" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="I50" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="J50">
-        <v>437.2</v>
+        <v>443.7</v>
       </c>
       <c r="K50">
-        <v>21.4</v>
+        <v>21.3</v>
       </c>
       <c r="L50">
         <v>5</v>
@@ -15943,13 +15937,13 @@
         <v>0</v>
       </c>
       <c r="T50" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="U50" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="V50" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="W50">
         <v>0.6667</v>
@@ -16066,7 +16060,7 @@
         <v>1.157</v>
       </c>
       <c r="BI50" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="BJ50">
         <v>1846</v>
@@ -16137,25 +16131,25 @@
         <v>129</v>
       </c>
       <c r="E51" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="F51" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="G51" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="H51" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="I51" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="J51">
-        <v>437.2</v>
+        <v>443.7</v>
       </c>
       <c r="K51">
-        <v>22.4</v>
+        <v>22.3</v>
       </c>
       <c r="L51">
         <v>5</v>
@@ -16182,13 +16176,13 @@
         <v>0</v>
       </c>
       <c r="T51" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="U51" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="V51" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="W51">
         <v>0.6667</v>
@@ -16305,7 +16299,7 @@
         <v>1.1689</v>
       </c>
       <c r="BI51" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="BJ51">
         <v>1474</v>
@@ -16376,25 +16370,25 @@
         <v>129</v>
       </c>
       <c r="E52" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="F52" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="G52" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="H52" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="I52" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="J52">
-        <v>437.2</v>
+        <v>443.7</v>
       </c>
       <c r="K52">
-        <v>23.4</v>
+        <v>23.3</v>
       </c>
       <c r="L52">
         <v>5</v>
@@ -16421,13 +16415,13 @@
         <v>0</v>
       </c>
       <c r="T52" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="U52" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="V52" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="W52">
         <v>0.6667</v>
@@ -16544,7 +16538,7 @@
         <v>1.1815</v>
       </c>
       <c r="BI52" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="BJ52">
         <v>1092</v>
@@ -16583,7 +16577,7 @@
         <v>185</v>
       </c>
       <c r="BV52">
-        <v>5.6</v>
+        <v>5.5</v>
       </c>
       <c r="BW52" t="s">
         <v>185</v>
@@ -16615,25 +16609,25 @@
         <v>129</v>
       </c>
       <c r="E53" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="F53" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="G53" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="H53" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="I53" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="J53">
-        <v>437.2</v>
+        <v>443.7</v>
       </c>
       <c r="K53">
-        <v>24.4</v>
+        <v>24.3</v>
       </c>
       <c r="L53">
         <v>5</v>
@@ -16660,13 +16654,13 @@
         <v>0</v>
       </c>
       <c r="T53" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="U53" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="V53" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="W53">
         <v>0.6667</v>
@@ -16783,7 +16777,7 @@
         <v>1.1915</v>
       </c>
       <c r="BI53" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="BJ53">
         <v>794</v>
@@ -16854,25 +16848,25 @@
         <v>130</v>
       </c>
       <c r="E54" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F54" t="s">
         <v>116</v>
       </c>
       <c r="G54" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="H54" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="I54" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="J54">
-        <v>324.7</v>
+        <v>331.3</v>
       </c>
       <c r="K54">
-        <v>21.4</v>
+        <v>21.3</v>
       </c>
       <c r="L54">
         <v>5</v>
@@ -16899,13 +16893,13 @@
         <v>81.2</v>
       </c>
       <c r="T54" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="U54" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="V54" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="W54">
         <v>0.6667</v>
@@ -16914,7 +16908,7 @@
         <v>14</v>
       </c>
       <c r="Y54">
-        <v>82.5</v>
+        <v>82.59999999999999</v>
       </c>
       <c r="Z54">
         <v>67.7</v>
@@ -17022,7 +17016,7 @@
         <v>1.1072</v>
       </c>
       <c r="BI54" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="BJ54">
         <v>3121</v>
@@ -17093,25 +17087,25 @@
         <v>130</v>
       </c>
       <c r="E55" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="F55" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="G55" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="H55" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="I55" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="J55">
-        <v>324.7</v>
+        <v>331.3</v>
       </c>
       <c r="K55">
-        <v>22.4</v>
+        <v>22.3</v>
       </c>
       <c r="L55">
         <v>5</v>
@@ -17138,13 +17132,13 @@
         <v>25</v>
       </c>
       <c r="T55" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="U55" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="V55" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="W55">
         <v>0.6667</v>
@@ -17261,7 +17255,7 @@
         <v>1.1089</v>
       </c>
       <c r="BI55" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="BJ55">
         <v>3058</v>
@@ -17332,25 +17326,25 @@
         <v>130</v>
       </c>
       <c r="E56" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="F56" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="G56" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="H56" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="I56" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="J56">
-        <v>324.7</v>
+        <v>331.3</v>
       </c>
       <c r="K56">
-        <v>23.4</v>
+        <v>23.3</v>
       </c>
       <c r="L56">
         <v>5</v>
@@ -17377,13 +17371,13 @@
         <v>25</v>
       </c>
       <c r="T56" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="U56" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="V56" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="W56">
         <v>0.6667</v>
@@ -17500,7 +17494,7 @@
         <v>1.1111</v>
       </c>
       <c r="BI56" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="BJ56">
         <v>2992</v>
@@ -17539,7 +17533,7 @@
         <v>185</v>
       </c>
       <c r="BV56">
-        <v>22</v>
+        <v>21.9</v>
       </c>
       <c r="BW56" t="s">
         <v>187</v>
@@ -17571,25 +17565,25 @@
         <v>130</v>
       </c>
       <c r="E57" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="F57" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="G57" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="H57" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="I57" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="J57">
-        <v>324.7</v>
+        <v>331.3</v>
       </c>
       <c r="K57">
-        <v>24.4</v>
+        <v>24.3</v>
       </c>
       <c r="L57">
         <v>5</v>
@@ -17616,13 +17610,13 @@
         <v>25</v>
       </c>
       <c r="T57" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="U57" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="V57" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="W57">
         <v>0.6667</v>
@@ -17631,7 +17625,7 @@
         <v>8.199999999999999</v>
       </c>
       <c r="Y57">
-        <v>84.59999999999999</v>
+        <v>84.7</v>
       </c>
       <c r="Z57">
         <v>67.59999999999999</v>
@@ -17739,7 +17733,7 @@
         <v>1.1131</v>
       </c>
       <c r="BI57" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="BJ57">
         <v>2928</v>
@@ -17810,25 +17804,25 @@
         <v>131</v>
       </c>
       <c r="E58" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F58" t="s">
         <v>117</v>
       </c>
       <c r="G58" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="H58" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="I58" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="J58">
-        <v>442.9</v>
+        <v>449.4</v>
       </c>
       <c r="K58">
-        <v>21.9</v>
+        <v>21.8</v>
       </c>
       <c r="L58">
         <v>5</v>
@@ -17855,13 +17849,13 @@
         <v>56.2</v>
       </c>
       <c r="T58" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="U58" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="V58" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="W58">
         <v>0.1667</v>
@@ -17978,7 +17972,7 @@
         <v>1.1875</v>
       </c>
       <c r="BI58" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="BJ58">
         <v>885</v>
@@ -18049,25 +18043,25 @@
         <v>131</v>
       </c>
       <c r="E59" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="F59" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="G59" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="H59" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="I59" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="J59">
-        <v>442.9</v>
+        <v>449.4</v>
       </c>
       <c r="K59">
-        <v>22.9</v>
+        <v>22.8</v>
       </c>
       <c r="L59">
         <v>5</v>
@@ -18094,13 +18088,13 @@
         <v>56.2</v>
       </c>
       <c r="T59" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="U59" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="V59" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="W59">
         <v>0.1667</v>
@@ -18169,7 +18163,7 @@
         <v>9.4</v>
       </c>
       <c r="AS59" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="AT59">
         <v>325.1</v>
@@ -18217,7 +18211,7 @@
         <v>1.1931</v>
       </c>
       <c r="BI59" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="BJ59">
         <v>720</v>
@@ -18288,25 +18282,25 @@
         <v>131</v>
       </c>
       <c r="E60" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="F60" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="G60" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="H60" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="I60" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="J60">
-        <v>442.9</v>
+        <v>449.4</v>
       </c>
       <c r="K60">
-        <v>23.9</v>
+        <v>23.8</v>
       </c>
       <c r="L60">
         <v>5</v>
@@ -18333,13 +18327,13 @@
         <v>56.2</v>
       </c>
       <c r="T60" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="U60" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="V60" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="W60">
         <v>0.1667</v>
@@ -18408,7 +18402,7 @@
         <v>8.6</v>
       </c>
       <c r="AS60" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="AT60">
         <v>332.6</v>
@@ -18456,7 +18450,7 @@
         <v>1.2008</v>
       </c>
       <c r="BI60" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="BJ60">
         <v>497</v>
@@ -18527,25 +18521,25 @@
         <v>131</v>
       </c>
       <c r="E61" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="F61" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="G61" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="H61" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="I61" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="J61">
-        <v>442.9</v>
+        <v>449.4</v>
       </c>
       <c r="K61">
-        <v>24.9</v>
+        <v>24.8</v>
       </c>
       <c r="L61">
         <v>5</v>
@@ -18572,13 +18566,13 @@
         <v>56.2</v>
       </c>
       <c r="T61" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="U61" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="V61" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="W61">
         <v>0.1667</v>
@@ -18647,7 +18641,7 @@
         <v>6.8</v>
       </c>
       <c r="AS61" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="AT61">
         <v>341.2</v>
@@ -18695,7 +18689,7 @@
         <v>1.2065</v>
       </c>
       <c r="BI61" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="BJ61">
         <v>335</v>
@@ -18734,7 +18728,7 @@
         <v>185</v>
       </c>
       <c r="BV61">
-        <v>13</v>
+        <v>12.9</v>
       </c>
       <c r="BW61" t="s">
         <v>185</v>
@@ -19280,7 +19274,7 @@
         <v>163</v>
       </c>
       <c r="G10">
-        <v>90.09999999999999</v>
+        <v>90.2</v>
       </c>
       <c r="H10">
         <v>5</v>

</xml_diff>

<commit_message>
Update MLB weather 2026-07-16 09:26 PM PT
</commit_message>
<xml_diff>
--- a/mlb_weather_professional_v4_2026_07_17.xlsx
+++ b/mlb_weather_professional_v4_2026_07_17.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1852" uniqueCount="364">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1852" uniqueCount="362">
   <si>
     <t>Date</t>
   </si>
@@ -587,46 +587,43 @@
     <t>MEDIUM</t>
   </si>
   <si>
-    <t>2026-07-16 09:24:25 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-16 09:24:26 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-16 09:24:27 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-16 09:24:28 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-16 09:24:29 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-16 09:24:33 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-16 09:24:34 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-16 09:24:35 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-16 09:24:36 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-16 09:24:37 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-16 09:24:38 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-16 09:24:39 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-16 09:24:40 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-16 09:24:41 PM PDT</t>
+    <t>2026-07-16 09:26:11 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-16 09:26:12 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-16 09:26:13 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-16 09:26:14 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-16 09:26:15 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-16 09:26:20 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-16 09:26:21 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-16 09:26:22 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-16 09:26:23 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-16 09:26:24 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-16 09:26:25 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-16 09:26:26 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-16 09:26:27 PM PDT</t>
   </si>
   <si>
     <t>Period</t>
@@ -959,46 +956,43 @@
     <t>10:10 PM PDT</t>
   </si>
   <si>
-    <t>2026-07-17 04:24:25 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-17 04:24:26 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-17 04:24:27 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-17 04:24:28 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-17 04:24:29 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-17 04:24:33 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-17 04:24:34 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-17 04:24:35 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-17 04:24:36 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-17 04:24:37 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-17 04:24:38 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-17 04:24:39 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-17 04:24:40 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-17 04:24:41 UTC</t>
+    <t>2026-07-17 04:26:11 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-17 04:26:12 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-17 04:26:13 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-17 04:26:14 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-17 04:26:15 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-17 04:26:20 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-17 04:26:21 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-17 04:26:22 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-17 04:26:23 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-17 04:26:24 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-17 04:26:25 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-17 04:26:26 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-17 04:26:27 UTC</t>
   </si>
   <si>
     <t>2026-07-16T19:01:48+00:00</t>
@@ -1913,7 +1907,7 @@
         <v>188</v>
       </c>
       <c r="AY2">
-        <v>562.6</v>
+        <v>564.4</v>
       </c>
       <c r="AZ2">
         <v>5</v>
@@ -2068,7 +2062,7 @@
         <v>189</v>
       </c>
       <c r="AY3">
-        <v>343</v>
+        <v>344.8</v>
       </c>
       <c r="AZ3">
         <v>5</v>
@@ -2223,7 +2217,7 @@
         <v>190</v>
       </c>
       <c r="AY4">
-        <v>562.7</v>
+        <v>564.4</v>
       </c>
       <c r="AZ4">
         <v>5</v>
@@ -2378,7 +2372,7 @@
         <v>191</v>
       </c>
       <c r="AY5">
-        <v>487.8</v>
+        <v>489.6</v>
       </c>
       <c r="AZ5">
         <v>5</v>
@@ -2533,7 +2527,7 @@
         <v>192</v>
       </c>
       <c r="AY6">
-        <v>331.9</v>
+        <v>333.6</v>
       </c>
       <c r="AZ6">
         <v>5</v>
@@ -2843,7 +2837,7 @@
         <v>194</v>
       </c>
       <c r="AY8">
-        <v>167.3</v>
+        <v>169.1</v>
       </c>
       <c r="AZ8">
         <v>5</v>
@@ -2995,10 +2989,10 @@
         <v>21.8</v>
       </c>
       <c r="AX9" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="AY9">
-        <v>63.2</v>
+        <v>65</v>
       </c>
       <c r="AZ9">
         <v>5</v>
@@ -3150,10 +3144,10 @@
         <v>15.8</v>
       </c>
       <c r="AX10" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="AY10">
-        <v>38.2</v>
+        <v>39.9</v>
       </c>
       <c r="AZ10">
         <v>5</v>
@@ -3305,10 +3299,10 @@
         <v>13.5</v>
       </c>
       <c r="AX11" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="AY11">
-        <v>12.4</v>
+        <v>14.2</v>
       </c>
       <c r="AZ11">
         <v>5</v>
@@ -3460,10 +3454,10 @@
         <v>8.699999999999999</v>
       </c>
       <c r="AX12" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="AY12">
-        <v>578.2</v>
+        <v>580</v>
       </c>
       <c r="AZ12">
         <v>5</v>
@@ -3615,10 +3609,10 @@
         <v>14.6</v>
       </c>
       <c r="AX13" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="AY13">
-        <v>38.3</v>
+        <v>40.1</v>
       </c>
       <c r="AZ13">
         <v>5</v>
@@ -3773,7 +3767,7 @@
         <v>199</v>
       </c>
       <c r="AY14">
-        <v>443.7</v>
+        <v>445.5</v>
       </c>
       <c r="AZ14">
         <v>5</v>
@@ -3928,7 +3922,7 @@
         <v>200</v>
       </c>
       <c r="AY15">
-        <v>331.3</v>
+        <v>333.1</v>
       </c>
       <c r="AZ15">
         <v>5</v>
@@ -4080,10 +4074,10 @@
         <v>18.1</v>
       </c>
       <c r="AX16" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="AY16">
-        <v>449.4</v>
+        <v>451.2</v>
       </c>
       <c r="AZ16">
         <v>5</v>
@@ -4205,211 +4199,211 @@
         <v>6</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>202</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>203</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>204</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>49</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>50</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="L1" s="1" t="s">
         <v>51</v>
       </c>
       <c r="M1" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="N1" s="1" t="s">
         <v>207</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>208</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>209</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>210</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>212</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>213</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="U1" s="1" t="s">
         <v>214</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="V1" s="1" t="s">
         <v>215</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="W1" s="1" t="s">
         <v>216</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="X1" s="1" t="s">
         <v>217</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>219</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>220</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AB1" s="1" t="s">
         <v>221</v>
       </c>
-      <c r="AB1" s="1" t="s">
+      <c r="AC1" s="1" t="s">
         <v>222</v>
       </c>
-      <c r="AC1" s="1" t="s">
+      <c r="AD1" s="1" t="s">
         <v>223</v>
       </c>
-      <c r="AD1" s="1" t="s">
+      <c r="AE1" s="1" t="s">
         <v>224</v>
       </c>
-      <c r="AE1" s="1" t="s">
+      <c r="AF1" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AF1" s="1" t="s">
+      <c r="AG1" s="1" t="s">
         <v>226</v>
       </c>
-      <c r="AG1" s="1" t="s">
+      <c r="AH1" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="AH1" s="1" t="s">
+      <c r="AI1" s="1" t="s">
         <v>228</v>
       </c>
-      <c r="AI1" s="1" t="s">
+      <c r="AJ1" s="1" t="s">
         <v>229</v>
       </c>
-      <c r="AJ1" s="1" t="s">
+      <c r="AK1" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="AK1" s="1" t="s">
+      <c r="AL1" s="1" t="s">
         <v>231</v>
       </c>
-      <c r="AL1" s="1" t="s">
+      <c r="AM1" s="1" t="s">
         <v>232</v>
       </c>
-      <c r="AM1" s="1" t="s">
+      <c r="AN1" s="1" t="s">
         <v>233</v>
       </c>
-      <c r="AN1" s="1" t="s">
+      <c r="AO1" s="1" t="s">
         <v>234</v>
       </c>
-      <c r="AO1" s="1" t="s">
+      <c r="AP1" s="1" t="s">
         <v>235</v>
       </c>
-      <c r="AP1" s="1" t="s">
+      <c r="AQ1" s="1" t="s">
         <v>236</v>
       </c>
-      <c r="AQ1" s="1" t="s">
+      <c r="AR1" s="1" t="s">
         <v>237</v>
       </c>
-      <c r="AR1" s="1" t="s">
+      <c r="AS1" s="1" t="s">
         <v>238</v>
       </c>
-      <c r="AS1" s="1" t="s">
+      <c r="AT1" s="1" t="s">
         <v>239</v>
       </c>
-      <c r="AT1" s="1" t="s">
+      <c r="AU1" s="1" t="s">
         <v>240</v>
       </c>
-      <c r="AU1" s="1" t="s">
+      <c r="AV1" s="1" t="s">
         <v>241</v>
       </c>
-      <c r="AV1" s="1" t="s">
+      <c r="AW1" s="1" t="s">
         <v>242</v>
       </c>
-      <c r="AW1" s="1" t="s">
+      <c r="AX1" s="1" t="s">
         <v>243</v>
       </c>
-      <c r="AX1" s="1" t="s">
+      <c r="AY1" s="1" t="s">
         <v>244</v>
       </c>
-      <c r="AY1" s="1" t="s">
+      <c r="AZ1" s="1" t="s">
         <v>245</v>
       </c>
-      <c r="AZ1" s="1" t="s">
+      <c r="BA1" s="1" t="s">
         <v>246</v>
       </c>
-      <c r="BA1" s="1" t="s">
+      <c r="BB1" s="1" t="s">
         <v>247</v>
       </c>
-      <c r="BB1" s="1" t="s">
+      <c r="BC1" s="1" t="s">
         <v>248</v>
       </c>
-      <c r="BC1" s="1" t="s">
+      <c r="BD1" s="1" t="s">
         <v>249</v>
       </c>
-      <c r="BD1" s="1" t="s">
+      <c r="BE1" s="1" t="s">
         <v>250</v>
       </c>
-      <c r="BE1" s="1" t="s">
+      <c r="BF1" s="1" t="s">
         <v>251</v>
       </c>
-      <c r="BF1" s="1" t="s">
+      <c r="BG1" s="1" t="s">
         <v>252</v>
       </c>
-      <c r="BG1" s="1" t="s">
+      <c r="BH1" s="1" t="s">
         <v>253</v>
       </c>
-      <c r="BH1" s="1" t="s">
+      <c r="BI1" s="1" t="s">
         <v>254</v>
       </c>
-      <c r="BI1" s="1" t="s">
+      <c r="BJ1" s="1" t="s">
         <v>255</v>
       </c>
-      <c r="BJ1" s="1" t="s">
+      <c r="BK1" s="1" t="s">
         <v>256</v>
       </c>
-      <c r="BK1" s="1" t="s">
+      <c r="BL1" s="1" t="s">
         <v>257</v>
       </c>
-      <c r="BL1" s="1" t="s">
+      <c r="BM1" s="1" t="s">
         <v>258</v>
       </c>
-      <c r="BM1" s="1" t="s">
+      <c r="BN1" s="1" t="s">
         <v>259</v>
       </c>
-      <c r="BN1" s="1" t="s">
+      <c r="BO1" s="1" t="s">
         <v>260</v>
       </c>
-      <c r="BO1" s="1" t="s">
+      <c r="BP1" s="1" t="s">
         <v>261</v>
       </c>
-      <c r="BP1" s="1" t="s">
+      <c r="BQ1" s="1" t="s">
         <v>262</v>
       </c>
-      <c r="BQ1" s="1" t="s">
+      <c r="BR1" s="1" t="s">
         <v>263</v>
       </c>
-      <c r="BR1" s="1" t="s">
+      <c r="BS1" s="1" t="s">
         <v>264</v>
       </c>
-      <c r="BS1" s="1" t="s">
+      <c r="BT1" s="1" t="s">
         <v>265</v>
       </c>
-      <c r="BT1" s="1" t="s">
+      <c r="BU1" s="1" t="s">
         <v>266</v>
-      </c>
-      <c r="BU1" s="1" t="s">
-        <v>267</v>
       </c>
       <c r="BV1" s="1" t="s">
         <v>48</v>
@@ -4418,16 +4412,16 @@
         <v>47</v>
       </c>
       <c r="BX1" s="1" t="s">
+        <v>267</v>
+      </c>
+      <c r="BY1" s="1" t="s">
         <v>268</v>
       </c>
-      <c r="BY1" s="1" t="s">
+      <c r="BZ1" s="1" t="s">
         <v>269</v>
       </c>
-      <c r="BZ1" s="1" t="s">
+      <c r="CA1" s="1" t="s">
         <v>270</v>
-      </c>
-      <c r="CA1" s="1" t="s">
-        <v>271</v>
       </c>
     </row>
     <row r="2" spans="1:79">
@@ -4444,25 +4438,25 @@
         <v>118</v>
       </c>
       <c r="E2" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="F2" t="s">
         <v>106</v>
       </c>
       <c r="G2" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="H2" t="s">
         <v>188</v>
       </c>
       <c r="I2" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="J2">
-        <v>562.6</v>
+        <v>564.4</v>
       </c>
       <c r="K2">
-        <v>13.2</v>
+        <v>13.1</v>
       </c>
       <c r="L2">
         <v>5</v>
@@ -4489,13 +4483,13 @@
         <v>0</v>
       </c>
       <c r="T2" t="s">
+        <v>337</v>
+      </c>
+      <c r="U2" t="s">
+        <v>338</v>
+      </c>
+      <c r="V2" t="s">
         <v>339</v>
-      </c>
-      <c r="U2" t="s">
-        <v>340</v>
-      </c>
-      <c r="V2" t="s">
-        <v>341</v>
       </c>
       <c r="W2">
         <v>0.5833</v>
@@ -4612,7 +4606,7 @@
         <v>1.1658</v>
       </c>
       <c r="BI2" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="BJ2">
         <v>1595</v>
@@ -4683,25 +4677,25 @@
         <v>118</v>
       </c>
       <c r="E3" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F3" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="G3" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="H3" t="s">
         <v>188</v>
       </c>
       <c r="I3" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="J3">
-        <v>562.6</v>
+        <v>564.4</v>
       </c>
       <c r="K3">
-        <v>14.2</v>
+        <v>14.1</v>
       </c>
       <c r="L3">
         <v>5</v>
@@ -4728,13 +4722,13 @@
         <v>0</v>
       </c>
       <c r="T3" t="s">
+        <v>337</v>
+      </c>
+      <c r="U3" t="s">
         <v>339</v>
       </c>
-      <c r="U3" t="s">
-        <v>341</v>
-      </c>
       <c r="V3" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="W3">
         <v>0.5833</v>
@@ -4761,7 +4755,7 @@
         <v>0.6</v>
       </c>
       <c r="AE3" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="AF3">
         <v>84.5</v>
@@ -4851,7 +4845,7 @@
         <v>1.1623</v>
       </c>
       <c r="BI3" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="BJ3">
         <v>1703</v>
@@ -4922,25 +4916,25 @@
         <v>118</v>
       </c>
       <c r="E4" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="F4" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="G4" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="H4" t="s">
         <v>188</v>
       </c>
       <c r="I4" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="J4">
-        <v>562.6</v>
+        <v>564.4</v>
       </c>
       <c r="K4">
-        <v>15.2</v>
+        <v>15.1</v>
       </c>
       <c r="L4">
         <v>5</v>
@@ -4967,13 +4961,13 @@
         <v>0</v>
       </c>
       <c r="T4" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="U4" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="V4" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="W4">
         <v>0.5833</v>
@@ -5090,7 +5084,7 @@
         <v>1.1606</v>
       </c>
       <c r="BI4" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="BJ4">
         <v>1761</v>
@@ -5161,25 +5155,25 @@
         <v>118</v>
       </c>
       <c r="E5" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="F5" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="G5" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="H5" t="s">
         <v>188</v>
       </c>
       <c r="I5" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="J5">
-        <v>562.6</v>
+        <v>564.4</v>
       </c>
       <c r="K5">
-        <v>16.2</v>
+        <v>16.1</v>
       </c>
       <c r="L5">
         <v>5</v>
@@ -5206,13 +5200,13 @@
         <v>0</v>
       </c>
       <c r="T5" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="U5" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="V5" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="W5">
         <v>0.5833</v>
@@ -5329,7 +5323,7 @@
         <v>1.1603</v>
       </c>
       <c r="BI5" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="BJ5">
         <v>1772</v>
@@ -5400,25 +5394,25 @@
         <v>119</v>
       </c>
       <c r="E6" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="F6" t="s">
         <v>107</v>
       </c>
       <c r="G6" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="H6" t="s">
         <v>189</v>
       </c>
       <c r="I6" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="J6">
-        <v>343</v>
+        <v>344.8</v>
       </c>
       <c r="K6">
-        <v>18.7</v>
+        <v>18.6</v>
       </c>
       <c r="L6">
         <v>5</v>
@@ -5445,13 +5439,13 @@
         <v>0</v>
       </c>
       <c r="T6" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="U6" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="V6" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="W6">
         <v>0.0833</v>
@@ -5568,7 +5562,7 @@
         <v>1.156</v>
       </c>
       <c r="BI6" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="BJ6">
         <v>1880</v>
@@ -5639,25 +5633,25 @@
         <v>119</v>
       </c>
       <c r="E7" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F7" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="G7" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="H7" t="s">
         <v>189</v>
       </c>
       <c r="I7" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="J7">
-        <v>343</v>
+        <v>344.8</v>
       </c>
       <c r="K7">
-        <v>19.7</v>
+        <v>19.6</v>
       </c>
       <c r="L7">
         <v>5</v>
@@ -5684,13 +5678,13 @@
         <v>56.2</v>
       </c>
       <c r="T7" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="U7" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="V7" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="W7">
         <v>0.0833</v>
@@ -5759,7 +5753,7 @@
         <v>7</v>
       </c>
       <c r="AS7" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="AT7">
         <v>75.59999999999999</v>
@@ -5807,7 +5801,7 @@
         <v>1.1612</v>
       </c>
       <c r="BI7" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="BJ7">
         <v>1705</v>
@@ -5878,25 +5872,25 @@
         <v>119</v>
       </c>
       <c r="E8" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="F8" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="G8" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="H8" t="s">
         <v>189</v>
       </c>
       <c r="I8" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="J8">
-        <v>343</v>
+        <v>344.8</v>
       </c>
       <c r="K8">
-        <v>20.7</v>
+        <v>20.6</v>
       </c>
       <c r="L8">
         <v>5</v>
@@ -5923,13 +5917,13 @@
         <v>75</v>
       </c>
       <c r="T8" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="U8" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="V8" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="W8">
         <v>0.0833</v>
@@ -6046,7 +6040,7 @@
         <v>1.169</v>
       </c>
       <c r="BI8" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="BJ8">
         <v>1415</v>
@@ -6117,25 +6111,25 @@
         <v>119</v>
       </c>
       <c r="E9" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="F9" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="G9" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="H9" t="s">
         <v>189</v>
       </c>
       <c r="I9" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="J9">
-        <v>343</v>
+        <v>344.8</v>
       </c>
       <c r="K9">
-        <v>21.7</v>
+        <v>21.6</v>
       </c>
       <c r="L9">
         <v>5</v>
@@ -6162,13 +6156,13 @@
         <v>100</v>
       </c>
       <c r="T9" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="U9" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="V9" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="W9">
         <v>0.0833</v>
@@ -6237,7 +6231,7 @@
         <v>9.4</v>
       </c>
       <c r="AS9" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="AT9">
         <v>150.3</v>
@@ -6285,7 +6279,7 @@
         <v>1.1726</v>
       </c>
       <c r="BI9" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="BJ9">
         <v>1288</v>
@@ -6356,25 +6350,25 @@
         <v>118</v>
       </c>
       <c r="E10" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="F10" t="s">
         <v>108</v>
       </c>
       <c r="G10" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="H10" t="s">
         <v>190</v>
       </c>
       <c r="I10" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="J10">
-        <v>562.7</v>
+        <v>564.4</v>
       </c>
       <c r="K10">
-        <v>18.8</v>
+        <v>18.7</v>
       </c>
       <c r="L10">
         <v>5</v>
@@ -6401,13 +6395,13 @@
         <v>25</v>
       </c>
       <c r="T10" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="U10" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="V10" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="W10">
         <v>0.1667</v>
@@ -6524,7 +6518,7 @@
         <v>1.1688</v>
       </c>
       <c r="BI10" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="BJ10">
         <v>1505</v>
@@ -6595,25 +6589,25 @@
         <v>118</v>
       </c>
       <c r="E11" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F11" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="G11" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="H11" t="s">
         <v>190</v>
       </c>
       <c r="I11" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="J11">
-        <v>562.7</v>
+        <v>564.4</v>
       </c>
       <c r="K11">
-        <v>19.8</v>
+        <v>19.7</v>
       </c>
       <c r="L11">
         <v>5</v>
@@ -6640,13 +6634,13 @@
         <v>81.2</v>
       </c>
       <c r="T11" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="U11" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="V11" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="W11">
         <v>0.1667</v>
@@ -6715,7 +6709,7 @@
         <v>8.699999999999999</v>
       </c>
       <c r="AS11" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="AT11">
         <v>316.6</v>
@@ -6763,7 +6757,7 @@
         <v>1.1761</v>
       </c>
       <c r="BI11" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="BJ11">
         <v>1275</v>
@@ -6834,25 +6828,25 @@
         <v>118</v>
       </c>
       <c r="E12" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="F12" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="G12" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="H12" t="s">
         <v>190</v>
       </c>
       <c r="I12" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="J12">
-        <v>562.7</v>
+        <v>564.4</v>
       </c>
       <c r="K12">
-        <v>20.8</v>
+        <v>20.7</v>
       </c>
       <c r="L12">
         <v>5</v>
@@ -6879,13 +6873,13 @@
         <v>81.2</v>
       </c>
       <c r="T12" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="U12" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="V12" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="W12">
         <v>0.1667</v>
@@ -6894,7 +6888,7 @@
         <v>6.4</v>
       </c>
       <c r="Y12">
-        <v>91.2</v>
+        <v>91.3</v>
       </c>
       <c r="Z12">
         <v>50.7</v>
@@ -6912,7 +6906,7 @@
         <v>0.6</v>
       </c>
       <c r="AE12" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="AF12">
         <v>74.90000000000001</v>
@@ -7002,7 +6996,7 @@
         <v>1.1831</v>
       </c>
       <c r="BI12" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="BJ12">
         <v>1049</v>
@@ -7073,25 +7067,25 @@
         <v>118</v>
       </c>
       <c r="E13" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="F13" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="G13" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="H13" t="s">
         <v>190</v>
       </c>
       <c r="I13" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="J13">
-        <v>562.7</v>
+        <v>564.4</v>
       </c>
       <c r="K13">
-        <v>21.8</v>
+        <v>21.7</v>
       </c>
       <c r="L13">
         <v>5</v>
@@ -7118,13 +7112,13 @@
         <v>81.2</v>
       </c>
       <c r="T13" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="U13" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="V13" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="W13">
         <v>0.1667</v>
@@ -7193,7 +7187,7 @@
         <v>7.2</v>
       </c>
       <c r="AS13" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="AT13">
         <v>144.5</v>
@@ -7241,7 +7235,7 @@
         <v>1.189</v>
       </c>
       <c r="BI13" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="BJ13">
         <v>873</v>
@@ -7312,25 +7306,25 @@
         <v>120</v>
       </c>
       <c r="E14" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="F14" t="s">
         <v>108</v>
       </c>
       <c r="G14" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="H14" t="s">
         <v>191</v>
       </c>
       <c r="I14" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="J14">
-        <v>487.8</v>
+        <v>489.6</v>
       </c>
       <c r="K14">
-        <v>18.8</v>
+        <v>18.7</v>
       </c>
       <c r="L14">
         <v>5</v>
@@ -7357,13 +7351,13 @@
         <v>56.2</v>
       </c>
       <c r="T14" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="U14" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="V14" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="W14">
         <v>0.1667</v>
@@ -7480,7 +7474,7 @@
         <v>1.1393</v>
       </c>
       <c r="BI14" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="BJ14">
         <v>2273</v>
@@ -7551,25 +7545,25 @@
         <v>120</v>
       </c>
       <c r="E15" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F15" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="G15" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="H15" t="s">
         <v>191</v>
       </c>
       <c r="I15" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="J15">
-        <v>487.8</v>
+        <v>489.6</v>
       </c>
       <c r="K15">
-        <v>19.8</v>
+        <v>19.7</v>
       </c>
       <c r="L15">
         <v>5</v>
@@ -7596,13 +7590,13 @@
         <v>56.2</v>
       </c>
       <c r="T15" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="U15" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="V15" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="W15">
         <v>0.1667</v>
@@ -7671,7 +7665,7 @@
         <v>5.8</v>
       </c>
       <c r="AS15" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="AT15">
         <v>78.2</v>
@@ -7719,7 +7713,7 @@
         <v>1.1418</v>
       </c>
       <c r="BI15" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="BJ15">
         <v>2187</v>
@@ -7790,25 +7784,25 @@
         <v>120</v>
       </c>
       <c r="E16" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="F16" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="G16" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="H16" t="s">
         <v>191</v>
       </c>
       <c r="I16" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="J16">
-        <v>487.8</v>
+        <v>489.6</v>
       </c>
       <c r="K16">
-        <v>20.8</v>
+        <v>20.7</v>
       </c>
       <c r="L16">
         <v>5</v>
@@ -7835,13 +7829,13 @@
         <v>56.2</v>
       </c>
       <c r="T16" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="U16" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="V16" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="W16">
         <v>0.1667</v>
@@ -7910,7 +7904,7 @@
         <v>6</v>
       </c>
       <c r="AS16" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="AT16">
         <v>133.6</v>
@@ -7958,7 +7952,7 @@
         <v>1.1467</v>
       </c>
       <c r="BI16" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="BJ16">
         <v>2033</v>
@@ -8029,25 +8023,25 @@
         <v>120</v>
       </c>
       <c r="E17" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="F17" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="G17" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="H17" t="s">
         <v>191</v>
       </c>
       <c r="I17" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="J17">
-        <v>487.8</v>
+        <v>489.6</v>
       </c>
       <c r="K17">
-        <v>21.8</v>
+        <v>21.7</v>
       </c>
       <c r="L17">
         <v>5</v>
@@ -8074,13 +8068,13 @@
         <v>0</v>
       </c>
       <c r="T17" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="U17" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="V17" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="W17">
         <v>0.1667</v>
@@ -8197,7 +8191,7 @@
         <v>1.1488</v>
       </c>
       <c r="BI17" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="BJ17">
         <v>1977</v>
@@ -8268,22 +8262,22 @@
         <v>121</v>
       </c>
       <c r="E18" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="F18" t="s">
         <v>109</v>
       </c>
       <c r="G18" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="H18" t="s">
         <v>192</v>
       </c>
       <c r="I18" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="J18">
-        <v>331.9</v>
+        <v>333.6</v>
       </c>
       <c r="K18">
         <v>18.8</v>
@@ -8313,13 +8307,13 @@
         <v>0</v>
       </c>
       <c r="T18" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="U18" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="V18" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="W18">
         <v>0.25</v>
@@ -8436,7 +8430,7 @@
         <v>1.123</v>
       </c>
       <c r="BI18" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="BJ18">
         <v>2642</v>
@@ -8507,22 +8501,22 @@
         <v>121</v>
       </c>
       <c r="E19" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F19" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="G19" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="H19" t="s">
         <v>192</v>
       </c>
       <c r="I19" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="J19">
-        <v>331.9</v>
+        <v>333.6</v>
       </c>
       <c r="K19">
         <v>19.8</v>
@@ -8552,13 +8546,13 @@
         <v>0</v>
       </c>
       <c r="T19" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="U19" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="V19" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="W19">
         <v>0.25</v>
@@ -8675,7 +8669,7 @@
         <v>1.1261</v>
       </c>
       <c r="BI19" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="BJ19">
         <v>2547</v>
@@ -8746,22 +8740,22 @@
         <v>121</v>
       </c>
       <c r="E20" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="F20" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="G20" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="H20" t="s">
         <v>192</v>
       </c>
       <c r="I20" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="J20">
-        <v>331.9</v>
+        <v>333.6</v>
       </c>
       <c r="K20">
         <v>20.8</v>
@@ -8791,13 +8785,13 @@
         <v>0</v>
       </c>
       <c r="T20" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="U20" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="V20" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="W20">
         <v>0.25</v>
@@ -8866,7 +8860,7 @@
         <v>14.4</v>
       </c>
       <c r="AS20" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="AT20">
         <v>305.7</v>
@@ -8914,7 +8908,7 @@
         <v>1.1303</v>
       </c>
       <c r="BI20" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="BJ20">
         <v>2417</v>
@@ -8953,7 +8947,7 @@
         <v>185</v>
       </c>
       <c r="BV20">
-        <v>3.7</v>
+        <v>3.6</v>
       </c>
       <c r="BW20" t="s">
         <v>185</v>
@@ -8985,22 +8979,22 @@
         <v>121</v>
       </c>
       <c r="E21" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="F21" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="G21" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="H21" t="s">
         <v>192</v>
       </c>
       <c r="I21" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="J21">
-        <v>331.9</v>
+        <v>333.6</v>
       </c>
       <c r="K21">
         <v>21.8</v>
@@ -9030,13 +9024,13 @@
         <v>0</v>
       </c>
       <c r="T21" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="U21" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="V21" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="W21">
         <v>0.25</v>
@@ -9105,7 +9099,7 @@
         <v>12.1</v>
       </c>
       <c r="AS21" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="AT21">
         <v>307.5</v>
@@ -9153,7 +9147,7 @@
         <v>1.1347</v>
       </c>
       <c r="BI21" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="BJ21">
         <v>2283</v>
@@ -9224,13 +9218,13 @@
         <v>122</v>
       </c>
       <c r="E22" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="F22" t="s">
         <v>109</v>
       </c>
       <c r="G22" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="H22" t="s">
         <v>193</v>
@@ -9266,13 +9260,13 @@
         <v>0</v>
       </c>
       <c r="T22" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="U22" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="V22" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="W22">
         <v>0.25</v>
@@ -9389,7 +9383,7 @@
         <v>1.171</v>
       </c>
       <c r="BI22" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="BJ22">
         <v>1338</v>
@@ -9457,13 +9451,13 @@
         <v>122</v>
       </c>
       <c r="E23" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F23" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="G23" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="H23" t="s">
         <v>193</v>
@@ -9499,13 +9493,13 @@
         <v>56.2</v>
       </c>
       <c r="T23" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="U23" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="V23" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="W23">
         <v>0.25</v>
@@ -9532,7 +9526,7 @@
         <v>0.2</v>
       </c>
       <c r="AE23" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="AF23">
         <v>73.8</v>
@@ -9622,7 +9616,7 @@
         <v>1.1724</v>
       </c>
       <c r="BI23" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="BJ23">
         <v>1295</v>
@@ -9690,13 +9684,13 @@
         <v>122</v>
       </c>
       <c r="E24" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="F24" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="G24" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="H24" t="s">
         <v>193</v>
@@ -9732,13 +9726,13 @@
         <v>56.2</v>
       </c>
       <c r="T24" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="U24" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="V24" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="W24">
         <v>0.25</v>
@@ -9855,7 +9849,7 @@
         <v>1.1749</v>
       </c>
       <c r="BI24" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="BJ24">
         <v>1218</v>
@@ -9923,13 +9917,13 @@
         <v>122</v>
       </c>
       <c r="E25" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="F25" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="G25" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="H25" t="s">
         <v>193</v>
@@ -9965,13 +9959,13 @@
         <v>56.2</v>
       </c>
       <c r="T25" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="U25" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="V25" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="W25">
         <v>0.25</v>
@@ -10040,7 +10034,7 @@
         <v>5.7</v>
       </c>
       <c r="AS25" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="AT25">
         <v>76.8</v>
@@ -10088,7 +10082,7 @@
         <v>1.1748</v>
       </c>
       <c r="BI25" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="BJ25">
         <v>1226</v>
@@ -10156,25 +10150,25 @@
         <v>123</v>
       </c>
       <c r="E26" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="F26" t="s">
         <v>110</v>
       </c>
       <c r="G26" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="H26" t="s">
         <v>194</v>
       </c>
       <c r="I26" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="J26">
-        <v>167.3</v>
+        <v>169.1</v>
       </c>
       <c r="K26">
-        <v>19.3</v>
+        <v>19.2</v>
       </c>
       <c r="L26">
         <v>5</v>
@@ -10201,13 +10195,13 @@
         <v>100</v>
       </c>
       <c r="T26" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="U26" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="V26" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="W26">
         <v>0.6667</v>
@@ -10324,7 +10318,7 @@
         <v>1.1896</v>
       </c>
       <c r="BI26" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="BJ26">
         <v>858</v>
@@ -10360,7 +10354,7 @@
         <v>0</v>
       </c>
       <c r="BU26" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="BV26">
         <v>9.6</v>
@@ -10395,25 +10389,25 @@
         <v>123</v>
       </c>
       <c r="E27" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F27" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="G27" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="H27" t="s">
         <v>194</v>
       </c>
       <c r="I27" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="J27">
-        <v>167.3</v>
+        <v>169.1</v>
       </c>
       <c r="K27">
-        <v>20.3</v>
+        <v>20.2</v>
       </c>
       <c r="L27">
         <v>5</v>
@@ -10440,13 +10434,13 @@
         <v>100</v>
       </c>
       <c r="T27" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="U27" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="V27" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="W27">
         <v>0.6667</v>
@@ -10473,7 +10467,7 @@
         <v>0.5</v>
       </c>
       <c r="AE27" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="AF27">
         <v>84.59999999999999</v>
@@ -10563,7 +10557,7 @@
         <v>1.1268</v>
       </c>
       <c r="BI27" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="BJ27">
         <v>2568</v>
@@ -10634,25 +10628,25 @@
         <v>123</v>
       </c>
       <c r="E28" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="F28" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="G28" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="H28" t="s">
         <v>194</v>
       </c>
       <c r="I28" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="J28">
-        <v>167.3</v>
+        <v>169.1</v>
       </c>
       <c r="K28">
-        <v>21.3</v>
+        <v>21.2</v>
       </c>
       <c r="L28">
         <v>5</v>
@@ -10679,13 +10673,13 @@
         <v>0</v>
       </c>
       <c r="T28" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="U28" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="V28" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="W28">
         <v>0.6667</v>
@@ -10712,7 +10706,7 @@
         <v>0.5</v>
       </c>
       <c r="AE28" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="AF28">
         <v>82.40000000000001</v>
@@ -10802,7 +10796,7 @@
         <v>1.1311</v>
       </c>
       <c r="BI28" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="BJ28">
         <v>2428</v>
@@ -10873,25 +10867,25 @@
         <v>123</v>
       </c>
       <c r="E29" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="F29" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="G29" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="H29" t="s">
         <v>194</v>
       </c>
       <c r="I29" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="J29">
-        <v>167.3</v>
+        <v>169.1</v>
       </c>
       <c r="K29">
-        <v>22.3</v>
+        <v>22.2</v>
       </c>
       <c r="L29">
         <v>5</v>
@@ -10918,13 +10912,13 @@
         <v>0</v>
       </c>
       <c r="T29" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="U29" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="V29" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="W29">
         <v>0.6667</v>
@@ -11041,7 +11035,7 @@
         <v>1.1348</v>
       </c>
       <c r="BI29" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="BJ29">
         <v>2316</v>
@@ -11112,25 +11106,25 @@
         <v>124</v>
       </c>
       <c r="E30" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="F30" t="s">
         <v>111</v>
       </c>
       <c r="G30" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="H30" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="I30" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="J30">
-        <v>63.2</v>
+        <v>65</v>
       </c>
       <c r="K30">
-        <v>19.7</v>
+        <v>19.6</v>
       </c>
       <c r="L30">
         <v>5</v>
@@ -11157,13 +11151,13 @@
         <v>0</v>
       </c>
       <c r="T30" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="U30" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="V30" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="W30">
         <v>0.0833</v>
@@ -11280,7 +11274,7 @@
         <v>1.1497</v>
       </c>
       <c r="BI30" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="BJ30">
         <v>1889</v>
@@ -11351,25 +11345,25 @@
         <v>124</v>
       </c>
       <c r="E31" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F31" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="G31" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="H31" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="I31" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="J31">
-        <v>63.2</v>
+        <v>65</v>
       </c>
       <c r="K31">
-        <v>20.7</v>
+        <v>20.6</v>
       </c>
       <c r="L31">
         <v>5</v>
@@ -11396,13 +11390,13 @@
         <v>0</v>
       </c>
       <c r="T31" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="U31" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="V31" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="W31">
         <v>0.0833</v>
@@ -11519,7 +11513,7 @@
         <v>1.1518</v>
       </c>
       <c r="BI31" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="BJ31">
         <v>1821</v>
@@ -11590,25 +11584,25 @@
         <v>124</v>
       </c>
       <c r="E32" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="F32" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="G32" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="H32" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="I32" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="J32">
-        <v>63.2</v>
+        <v>65</v>
       </c>
       <c r="K32">
-        <v>21.7</v>
+        <v>21.6</v>
       </c>
       <c r="L32">
         <v>5</v>
@@ -11635,13 +11629,13 @@
         <v>0</v>
       </c>
       <c r="T32" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="U32" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="V32" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="W32">
         <v>0.0833</v>
@@ -11758,7 +11752,7 @@
         <v>1.1537</v>
       </c>
       <c r="BI32" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="BJ32">
         <v>1747</v>
@@ -11829,25 +11823,25 @@
         <v>124</v>
       </c>
       <c r="E33" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="F33" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="G33" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="H33" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="I33" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="J33">
-        <v>63.2</v>
+        <v>65</v>
       </c>
       <c r="K33">
-        <v>22.7</v>
+        <v>22.6</v>
       </c>
       <c r="L33">
         <v>5</v>
@@ -11874,13 +11868,13 @@
         <v>0</v>
       </c>
       <c r="T33" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="U33" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="V33" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="W33">
         <v>0.0833</v>
@@ -11907,7 +11901,7 @@
         <v>1.8</v>
       </c>
       <c r="AE33" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="AF33">
         <v>81.09999999999999</v>
@@ -11997,7 +11991,7 @@
         <v>1.1564</v>
       </c>
       <c r="BI33" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="BJ33">
         <v>1654</v>
@@ -12068,25 +12062,25 @@
         <v>125</v>
       </c>
       <c r="E34" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="F34" t="s">
         <v>112</v>
       </c>
       <c r="G34" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="H34" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="I34" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="J34">
-        <v>38.2</v>
+        <v>39.9</v>
       </c>
       <c r="K34">
-        <v>19.8</v>
+        <v>19.7</v>
       </c>
       <c r="L34">
         <v>5</v>
@@ -12113,13 +12107,13 @@
         <v>0</v>
       </c>
       <c r="T34" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="U34" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="V34" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="W34">
         <v>0.1667</v>
@@ -12236,7 +12230,7 @@
         <v>1.1896</v>
       </c>
       <c r="BI34" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="BJ34">
         <v>858</v>
@@ -12272,7 +12266,7 @@
         <v>0</v>
       </c>
       <c r="BU34" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="BV34">
         <v>13</v>
@@ -12307,25 +12301,25 @@
         <v>125</v>
       </c>
       <c r="E35" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F35" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="G35" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="H35" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="I35" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="J35">
-        <v>38.2</v>
+        <v>39.9</v>
       </c>
       <c r="K35">
-        <v>20.8</v>
+        <v>20.7</v>
       </c>
       <c r="L35">
         <v>5</v>
@@ -12352,13 +12346,13 @@
         <v>0</v>
       </c>
       <c r="T35" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="U35" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="V35" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="W35">
         <v>0.1667</v>
@@ -12475,7 +12469,7 @@
         <v>1.1575</v>
       </c>
       <c r="BI35" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="BJ35">
         <v>1621</v>
@@ -12546,25 +12540,25 @@
         <v>125</v>
       </c>
       <c r="E36" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="F36" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="G36" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="H36" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="I36" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="J36">
-        <v>38.2</v>
+        <v>39.9</v>
       </c>
       <c r="K36">
-        <v>21.8</v>
+        <v>21.7</v>
       </c>
       <c r="L36">
         <v>5</v>
@@ -12591,13 +12585,13 @@
         <v>0</v>
       </c>
       <c r="T36" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="U36" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="V36" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="W36">
         <v>0.1667</v>
@@ -12714,7 +12708,7 @@
         <v>1.1622</v>
       </c>
       <c r="BI36" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="BJ36">
         <v>1467</v>
@@ -12785,25 +12779,25 @@
         <v>125</v>
       </c>
       <c r="E37" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="F37" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="G37" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="H37" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="I37" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="J37">
-        <v>38.2</v>
+        <v>39.9</v>
       </c>
       <c r="K37">
-        <v>22.8</v>
+        <v>22.7</v>
       </c>
       <c r="L37">
         <v>5</v>
@@ -12830,13 +12824,13 @@
         <v>0</v>
       </c>
       <c r="T37" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="U37" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="V37" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="W37">
         <v>0.1667</v>
@@ -12953,7 +12947,7 @@
         <v>1.1646</v>
       </c>
       <c r="BI37" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="BJ37">
         <v>1385</v>
@@ -13024,25 +13018,25 @@
         <v>126</v>
       </c>
       <c r="E38" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="F38" t="s">
         <v>112</v>
       </c>
       <c r="G38" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="H38" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="I38" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="J38">
-        <v>12.4</v>
+        <v>14.2</v>
       </c>
       <c r="K38">
-        <v>19.8</v>
+        <v>19.7</v>
       </c>
       <c r="L38">
         <v>5</v>
@@ -13069,13 +13063,13 @@
         <v>0</v>
       </c>
       <c r="T38" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="U38" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="V38" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="W38">
         <v>0.1667</v>
@@ -13192,7 +13186,7 @@
         <v>1.1173</v>
       </c>
       <c r="BI38" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="BJ38">
         <v>2873</v>
@@ -13263,25 +13257,25 @@
         <v>126</v>
       </c>
       <c r="E39" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F39" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="G39" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="H39" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="I39" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="J39">
-        <v>12.4</v>
+        <v>14.2</v>
       </c>
       <c r="K39">
-        <v>20.8</v>
+        <v>20.7</v>
       </c>
       <c r="L39">
         <v>5</v>
@@ -13308,13 +13302,13 @@
         <v>0</v>
       </c>
       <c r="T39" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="U39" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="V39" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="W39">
         <v>0.1667</v>
@@ -13431,7 +13425,7 @@
         <v>1.1216</v>
       </c>
       <c r="BI39" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="BJ39">
         <v>2731</v>
@@ -13502,25 +13496,25 @@
         <v>126</v>
       </c>
       <c r="E40" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="F40" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="G40" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="H40" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="I40" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="J40">
-        <v>12.4</v>
+        <v>14.2</v>
       </c>
       <c r="K40">
-        <v>21.8</v>
+        <v>21.7</v>
       </c>
       <c r="L40">
         <v>5</v>
@@ -13547,13 +13541,13 @@
         <v>0</v>
       </c>
       <c r="T40" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="U40" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="V40" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="W40">
         <v>0.1667</v>
@@ -13670,7 +13664,7 @@
         <v>1.1259</v>
       </c>
       <c r="BI40" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="BJ40">
         <v>2592</v>
@@ -13741,25 +13735,25 @@
         <v>126</v>
       </c>
       <c r="E41" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="F41" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="G41" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="H41" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="I41" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="J41">
-        <v>12.4</v>
+        <v>14.2</v>
       </c>
       <c r="K41">
-        <v>22.8</v>
+        <v>22.7</v>
       </c>
       <c r="L41">
         <v>5</v>
@@ -13786,13 +13780,13 @@
         <v>0</v>
       </c>
       <c r="T41" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="U41" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="V41" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="W41">
         <v>0.1667</v>
@@ -13909,7 +13903,7 @@
         <v>1.13</v>
       </c>
       <c r="BI41" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="BJ41">
         <v>2461</v>
@@ -13980,25 +13974,25 @@
         <v>127</v>
       </c>
       <c r="E42" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="F42" t="s">
         <v>113</v>
       </c>
       <c r="G42" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="H42" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="I42" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="J42">
-        <v>578.2</v>
+        <v>580</v>
       </c>
       <c r="K42">
-        <v>20.3</v>
+        <v>20.2</v>
       </c>
       <c r="L42">
         <v>5</v>
@@ -14025,13 +14019,13 @@
         <v>75</v>
       </c>
       <c r="T42" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="U42" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="V42" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="W42">
         <v>0.6667</v>
@@ -14148,7 +14142,7 @@
         <v>0.9556</v>
       </c>
       <c r="BI42" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="BJ42">
         <v>8309</v>
@@ -14219,25 +14213,25 @@
         <v>127</v>
       </c>
       <c r="E43" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F43" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="G43" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="H43" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="I43" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="J43">
-        <v>578.2</v>
+        <v>580</v>
       </c>
       <c r="K43">
-        <v>21.3</v>
+        <v>21.2</v>
       </c>
       <c r="L43">
         <v>5</v>
@@ -14264,13 +14258,13 @@
         <v>75</v>
       </c>
       <c r="T43" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="U43" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="V43" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="W43">
         <v>0.6667</v>
@@ -14387,7 +14381,7 @@
         <v>0.9583</v>
       </c>
       <c r="BI43" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="BJ43">
         <v>8204</v>
@@ -14458,25 +14452,25 @@
         <v>127</v>
       </c>
       <c r="E44" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="F44" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="G44" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="H44" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="I44" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="J44">
-        <v>578.2</v>
+        <v>580</v>
       </c>
       <c r="K44">
-        <v>22.3</v>
+        <v>22.2</v>
       </c>
       <c r="L44">
         <v>5</v>
@@ -14503,13 +14497,13 @@
         <v>0</v>
       </c>
       <c r="T44" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="U44" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="V44" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="W44">
         <v>0.6667</v>
@@ -14626,7 +14620,7 @@
         <v>0.9641999999999999</v>
       </c>
       <c r="BI44" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="BJ44">
         <v>7979</v>
@@ -14697,25 +14691,25 @@
         <v>127</v>
       </c>
       <c r="E45" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="F45" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="G45" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="H45" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="I45" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="J45">
-        <v>578.2</v>
+        <v>580</v>
       </c>
       <c r="K45">
-        <v>23.3</v>
+        <v>23.2</v>
       </c>
       <c r="L45">
         <v>5</v>
@@ -14742,13 +14736,13 @@
         <v>0</v>
       </c>
       <c r="T45" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="U45" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="V45" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="W45">
         <v>0.6667</v>
@@ -14775,7 +14769,7 @@
         <v>4</v>
       </c>
       <c r="AE45" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="AF45">
         <v>84.09999999999999</v>
@@ -14817,7 +14811,7 @@
         <v>19.4</v>
       </c>
       <c r="AS45" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="AT45">
         <v>132.2</v>
@@ -14865,7 +14859,7 @@
         <v>0.9697</v>
       </c>
       <c r="BI45" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="BJ45">
         <v>7772</v>
@@ -14936,22 +14930,22 @@
         <v>128</v>
       </c>
       <c r="E46" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="F46" t="s">
         <v>114</v>
       </c>
       <c r="G46" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="H46" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="I46" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="J46">
-        <v>38.3</v>
+        <v>40.1</v>
       </c>
       <c r="K46">
         <v>21.2</v>
@@ -14981,13 +14975,13 @@
         <v>0</v>
       </c>
       <c r="T46" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="U46" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="V46" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="W46">
         <v>0.6333</v>
@@ -15104,7 +15098,7 @@
         <v>1.1717</v>
       </c>
       <c r="BI46" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="BJ46">
         <v>1281</v>
@@ -15175,22 +15169,22 @@
         <v>128</v>
       </c>
       <c r="E47" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F47" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="G47" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="H47" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="I47" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="J47">
-        <v>38.3</v>
+        <v>40.1</v>
       </c>
       <c r="K47">
         <v>22.2</v>
@@ -15220,13 +15214,13 @@
         <v>0</v>
       </c>
       <c r="T47" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="U47" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="V47" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="W47">
         <v>0.6333</v>
@@ -15343,7 +15337,7 @@
         <v>1.1783</v>
       </c>
       <c r="BI47" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="BJ47">
         <v>1087</v>
@@ -15414,22 +15408,22 @@
         <v>128</v>
       </c>
       <c r="E48" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="F48" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="G48" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="H48" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="I48" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="J48">
-        <v>38.3</v>
+        <v>40.1</v>
       </c>
       <c r="K48">
         <v>23.2</v>
@@ -15459,13 +15453,13 @@
         <v>0</v>
       </c>
       <c r="T48" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="U48" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="V48" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="W48">
         <v>0.6333</v>
@@ -15492,7 +15486,7 @@
         <v>0</v>
       </c>
       <c r="AE48" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="AF48">
         <v>72.09999999999999</v>
@@ -15582,7 +15576,7 @@
         <v>1.1839</v>
       </c>
       <c r="BI48" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="BJ48">
         <v>917</v>
@@ -15653,22 +15647,22 @@
         <v>128</v>
       </c>
       <c r="E49" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="F49" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="G49" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="H49" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="I49" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="J49">
-        <v>38.3</v>
+        <v>40.1</v>
       </c>
       <c r="K49">
         <v>24.2</v>
@@ -15698,13 +15692,13 @@
         <v>0</v>
       </c>
       <c r="T49" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="U49" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="V49" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="W49">
         <v>0.6333</v>
@@ -15821,7 +15815,7 @@
         <v>1.1875</v>
       </c>
       <c r="BI49" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="BJ49">
         <v>808</v>
@@ -15892,25 +15886,25 @@
         <v>129</v>
       </c>
       <c r="E50" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="F50" t="s">
         <v>115</v>
       </c>
       <c r="G50" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="H50" t="s">
         <v>199</v>
       </c>
       <c r="I50" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="J50">
-        <v>443.7</v>
+        <v>445.5</v>
       </c>
       <c r="K50">
-        <v>21.3</v>
+        <v>21.2</v>
       </c>
       <c r="L50">
         <v>5</v>
@@ -15937,13 +15931,13 @@
         <v>0</v>
       </c>
       <c r="T50" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="U50" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="V50" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="W50">
         <v>0.6667</v>
@@ -16060,7 +16054,7 @@
         <v>1.157</v>
       </c>
       <c r="BI50" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="BJ50">
         <v>1846</v>
@@ -16131,25 +16125,25 @@
         <v>129</v>
       </c>
       <c r="E51" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F51" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="G51" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="H51" t="s">
         <v>199</v>
       </c>
       <c r="I51" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="J51">
-        <v>443.7</v>
+        <v>445.5</v>
       </c>
       <c r="K51">
-        <v>22.3</v>
+        <v>22.2</v>
       </c>
       <c r="L51">
         <v>5</v>
@@ -16176,13 +16170,13 @@
         <v>0</v>
       </c>
       <c r="T51" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="U51" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="V51" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="W51">
         <v>0.6667</v>
@@ -16299,7 +16293,7 @@
         <v>1.1689</v>
       </c>
       <c r="BI51" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="BJ51">
         <v>1474</v>
@@ -16370,25 +16364,25 @@
         <v>129</v>
       </c>
       <c r="E52" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="F52" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="G52" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="H52" t="s">
         <v>199</v>
       </c>
       <c r="I52" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="J52">
-        <v>443.7</v>
+        <v>445.5</v>
       </c>
       <c r="K52">
-        <v>23.3</v>
+        <v>23.2</v>
       </c>
       <c r="L52">
         <v>5</v>
@@ -16415,13 +16409,13 @@
         <v>0</v>
       </c>
       <c r="T52" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="U52" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="V52" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="W52">
         <v>0.6667</v>
@@ -16538,7 +16532,7 @@
         <v>1.1815</v>
       </c>
       <c r="BI52" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="BJ52">
         <v>1092</v>
@@ -16609,25 +16603,25 @@
         <v>129</v>
       </c>
       <c r="E53" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="F53" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="G53" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="H53" t="s">
         <v>199</v>
       </c>
       <c r="I53" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="J53">
-        <v>443.7</v>
+        <v>445.5</v>
       </c>
       <c r="K53">
-        <v>24.3</v>
+        <v>24.2</v>
       </c>
       <c r="L53">
         <v>5</v>
@@ -16654,13 +16648,13 @@
         <v>0</v>
       </c>
       <c r="T53" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="U53" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="V53" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="W53">
         <v>0.6667</v>
@@ -16777,7 +16771,7 @@
         <v>1.1915</v>
       </c>
       <c r="BI53" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="BJ53">
         <v>794</v>
@@ -16848,25 +16842,25 @@
         <v>130</v>
       </c>
       <c r="E54" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="F54" t="s">
         <v>116</v>
       </c>
       <c r="G54" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="H54" t="s">
         <v>200</v>
       </c>
       <c r="I54" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="J54">
-        <v>331.3</v>
+        <v>333.1</v>
       </c>
       <c r="K54">
-        <v>21.3</v>
+        <v>21.2</v>
       </c>
       <c r="L54">
         <v>5</v>
@@ -16893,13 +16887,13 @@
         <v>81.2</v>
       </c>
       <c r="T54" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="U54" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="V54" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="W54">
         <v>0.6667</v>
@@ -17016,7 +17010,7 @@
         <v>1.1072</v>
       </c>
       <c r="BI54" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="BJ54">
         <v>3121</v>
@@ -17087,25 +17081,25 @@
         <v>130</v>
       </c>
       <c r="E55" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F55" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="G55" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="H55" t="s">
         <v>200</v>
       </c>
       <c r="I55" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="J55">
-        <v>331.3</v>
+        <v>333.1</v>
       </c>
       <c r="K55">
-        <v>22.3</v>
+        <v>22.2</v>
       </c>
       <c r="L55">
         <v>5</v>
@@ -17132,13 +17126,13 @@
         <v>25</v>
       </c>
       <c r="T55" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="U55" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="V55" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="W55">
         <v>0.6667</v>
@@ -17255,7 +17249,7 @@
         <v>1.1089</v>
       </c>
       <c r="BI55" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="BJ55">
         <v>3058</v>
@@ -17326,25 +17320,25 @@
         <v>130</v>
       </c>
       <c r="E56" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="F56" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="G56" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="H56" t="s">
         <v>200</v>
       </c>
       <c r="I56" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="J56">
-        <v>331.3</v>
+        <v>333.1</v>
       </c>
       <c r="K56">
-        <v>23.3</v>
+        <v>23.2</v>
       </c>
       <c r="L56">
         <v>5</v>
@@ -17371,13 +17365,13 @@
         <v>25</v>
       </c>
       <c r="T56" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="U56" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="V56" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="W56">
         <v>0.6667</v>
@@ -17494,7 +17488,7 @@
         <v>1.1111</v>
       </c>
       <c r="BI56" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="BJ56">
         <v>2992</v>
@@ -17565,25 +17559,25 @@
         <v>130</v>
       </c>
       <c r="E57" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="F57" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="G57" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="H57" t="s">
         <v>200</v>
       </c>
       <c r="I57" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="J57">
-        <v>331.3</v>
+        <v>333.1</v>
       </c>
       <c r="K57">
-        <v>24.3</v>
+        <v>24.2</v>
       </c>
       <c r="L57">
         <v>5</v>
@@ -17610,13 +17604,13 @@
         <v>25</v>
       </c>
       <c r="T57" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="U57" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="V57" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="W57">
         <v>0.6667</v>
@@ -17733,7 +17727,7 @@
         <v>1.1131</v>
       </c>
       <c r="BI57" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="BJ57">
         <v>2928</v>
@@ -17804,25 +17798,25 @@
         <v>131</v>
       </c>
       <c r="E58" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="F58" t="s">
         <v>117</v>
       </c>
       <c r="G58" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="H58" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="I58" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="J58">
-        <v>449.4</v>
+        <v>451.2</v>
       </c>
       <c r="K58">
-        <v>21.8</v>
+        <v>21.7</v>
       </c>
       <c r="L58">
         <v>5</v>
@@ -17849,13 +17843,13 @@
         <v>56.2</v>
       </c>
       <c r="T58" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="U58" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="V58" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="W58">
         <v>0.1667</v>
@@ -17972,7 +17966,7 @@
         <v>1.1875</v>
       </c>
       <c r="BI58" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="BJ58">
         <v>885</v>
@@ -18043,25 +18037,25 @@
         <v>131</v>
       </c>
       <c r="E59" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F59" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="G59" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="H59" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="I59" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="J59">
-        <v>449.4</v>
+        <v>451.2</v>
       </c>
       <c r="K59">
-        <v>22.8</v>
+        <v>22.7</v>
       </c>
       <c r="L59">
         <v>5</v>
@@ -18088,13 +18082,13 @@
         <v>56.2</v>
       </c>
       <c r="T59" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="U59" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="V59" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="W59">
         <v>0.1667</v>
@@ -18163,7 +18157,7 @@
         <v>9.4</v>
       </c>
       <c r="AS59" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="AT59">
         <v>325.1</v>
@@ -18211,7 +18205,7 @@
         <v>1.1931</v>
       </c>
       <c r="BI59" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="BJ59">
         <v>720</v>
@@ -18282,25 +18276,25 @@
         <v>131</v>
       </c>
       <c r="E60" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="F60" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="G60" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="H60" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="I60" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="J60">
-        <v>449.4</v>
+        <v>451.2</v>
       </c>
       <c r="K60">
-        <v>23.8</v>
+        <v>23.7</v>
       </c>
       <c r="L60">
         <v>5</v>
@@ -18327,13 +18321,13 @@
         <v>56.2</v>
       </c>
       <c r="T60" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="U60" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="V60" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="W60">
         <v>0.1667</v>
@@ -18402,7 +18396,7 @@
         <v>8.6</v>
       </c>
       <c r="AS60" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="AT60">
         <v>332.6</v>
@@ -18450,7 +18444,7 @@
         <v>1.2008</v>
       </c>
       <c r="BI60" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="BJ60">
         <v>497</v>
@@ -18521,25 +18515,25 @@
         <v>131</v>
       </c>
       <c r="E61" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="F61" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="G61" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="H61" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="I61" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="J61">
-        <v>449.4</v>
+        <v>451.2</v>
       </c>
       <c r="K61">
-        <v>24.8</v>
+        <v>24.7</v>
       </c>
       <c r="L61">
         <v>5</v>
@@ -18566,13 +18560,13 @@
         <v>56.2</v>
       </c>
       <c r="T61" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="U61" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="V61" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="W61">
         <v>0.1667</v>
@@ -18641,7 +18635,7 @@
         <v>6.8</v>
       </c>
       <c r="AS61" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="AT61">
         <v>341.2</v>
@@ -18689,7 +18683,7 @@
         <v>1.2065</v>
       </c>
       <c r="BI61" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="BJ61">
         <v>335</v>

</xml_diff>